<commit_message>
Añadiendo admin, pass nueva
</commit_message>
<xml_diff>
--- a/apiService/Plantilla-modelo.xlsx
+++ b/apiService/Plantilla-modelo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollo-software\reporte-obras-main\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollo-software\reporte-obras-main\apiService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D3F1B06-91AD-4EED-A0CE-FCA62D454841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BE6827-62F7-408F-993E-FDBF619E2ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="947" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1443,7 +1443,7 @@
     <t xml:space="preserve">2.2  Comprobar bomba grupo presión 2:          </t>
   </si>
   <si>
-    <t>4.5 Verificar seguridades (FOTOS del cuadro antes y después) prueba nueva</t>
+    <t>4.5 Verificar seguridades (FOTOS del cuadro antes y después) prueba nueva 2</t>
   </si>
 </sst>
 </file>
@@ -1684,9 +1684,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1696,6 +1693,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1705,8 +1708,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1734,15 +1743,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -2122,13 +2122,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -2158,13 +2158,13 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="36" t="s">
+      <c r="D5" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="42"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -2454,13 +2454,13 @@
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="42" t="s">
+      <c r="D27" s="43" t="s">
         <v>162</v>
       </c>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
+      <c r="E27" s="44"/>
+      <c r="F27" s="44"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="45"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
@@ -2532,25 +2532,25 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="36" t="s">
+      <c r="D33" s="40" t="s">
         <v>156</v>
       </c>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="37"/>
-      <c r="H33" s="38"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="42"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="14"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="39" t="s">
+      <c r="D34" s="36" t="s">
         <v>242</v>
       </c>
-      <c r="E34" s="40"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="41"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="38"/>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -2610,13 +2610,13 @@
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="39" t="s">
+      <c r="D39" s="36" t="s">
         <v>241</v>
       </c>
-      <c r="E39" s="40"/>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="41"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="37"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="38"/>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -2769,32 +2769,6 @@
     <row r="282" ht="45" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D16:H16"/>
@@ -2811,6 +2785,32 @@
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D43:H43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3082,6 +3082,13 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="D4:H4"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D8:H8"/>
@@ -3094,13 +3101,6 @@
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="D4:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3143,13 +3143,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -3167,49 +3167,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="38"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="42"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="36" t="s">
+      <c r="D5" s="40" t="s">
         <v>365</v>
       </c>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="42"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="36" t="s">
+      <c r="D6" s="40" t="s">
         <v>366</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="38"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="42"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -3401,85 +3401,85 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="39" t="s">
+      <c r="D22" s="36" t="s">
         <v>371</v>
       </c>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="41"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="38"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="39" t="s">
+      <c r="D23" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="41"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="38"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="39" t="s">
+      <c r="D24" s="36" t="s">
         <v>374</v>
       </c>
-      <c r="E24" s="40"/>
-      <c r="F24" s="40"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="41"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="38"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="39" t="s">
+      <c r="D25" s="36" t="s">
         <v>375</v>
       </c>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="41"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="38"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="39" t="s">
+      <c r="D26" s="36" t="s">
         <v>373</v>
       </c>
-      <c r="E26" s="40"/>
-      <c r="F26" s="40"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="41"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="38"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="12"/>
-      <c r="D27" s="39" t="s">
+      <c r="D27" s="36" t="s">
         <v>372</v>
       </c>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="41"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="38"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="12"/>
-      <c r="D28" s="39" t="s">
+      <c r="D28" s="36" t="s">
         <v>231</v>
       </c>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="41"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="38"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3515,13 +3515,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="39" t="s">
+      <c r="D31" s="36" t="s">
         <v>376</v>
       </c>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="41"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="38"/>
     </row>
     <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -3689,13 +3689,13 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="36" t="s">
+      <c r="D44" s="40" t="s">
         <v>102</v>
       </c>
-      <c r="E44" s="37"/>
-      <c r="F44" s="37"/>
-      <c r="G44" s="37"/>
-      <c r="H44" s="38"/>
+      <c r="E44" s="41"/>
+      <c r="F44" s="41"/>
+      <c r="G44" s="41"/>
+      <c r="H44" s="42"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
@@ -3713,25 +3713,25 @@
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
-      <c r="D46" s="36" t="s">
+      <c r="D46" s="40" t="s">
         <v>378</v>
       </c>
-      <c r="E46" s="37"/>
-      <c r="F46" s="37"/>
-      <c r="G46" s="37"/>
-      <c r="H46" s="38"/>
+      <c r="E46" s="41"/>
+      <c r="F46" s="41"/>
+      <c r="G46" s="41"/>
+      <c r="H46" s="42"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="36" t="s">
+      <c r="D47" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="E47" s="37"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="37"/>
-      <c r="H47" s="38"/>
+      <c r="E47" s="41"/>
+      <c r="F47" s="41"/>
+      <c r="G47" s="41"/>
+      <c r="H47" s="42"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3875,13 +3875,13 @@
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
-      <c r="D58" s="42" t="s">
+      <c r="D58" s="43" t="s">
         <v>114</v>
       </c>
-      <c r="E58" s="43"/>
-      <c r="F58" s="43"/>
-      <c r="G58" s="43"/>
-      <c r="H58" s="44"/>
+      <c r="E58" s="44"/>
+      <c r="F58" s="44"/>
+      <c r="G58" s="44"/>
+      <c r="H58" s="45"/>
     </row>
     <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
@@ -4305,6 +4305,79 @@
     </row>
   </sheetData>
   <mergeCells count="89">
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D73:H73"/>
+    <mergeCell ref="D62:H62"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="D90:H90"/>
+    <mergeCell ref="D91:H91"/>
+    <mergeCell ref="D86:H86"/>
+    <mergeCell ref="D75:H75"/>
+    <mergeCell ref="D76:H76"/>
+    <mergeCell ref="D77:H77"/>
+    <mergeCell ref="D78:H78"/>
+    <mergeCell ref="D79:H79"/>
+    <mergeCell ref="D80:H80"/>
+    <mergeCell ref="D81:H81"/>
+    <mergeCell ref="D82:H82"/>
+    <mergeCell ref="D83:H83"/>
+    <mergeCell ref="D84:H84"/>
+    <mergeCell ref="D85:H85"/>
     <mergeCell ref="D31:H31"/>
     <mergeCell ref="D36:H36"/>
     <mergeCell ref="D87:H87"/>
@@ -4321,79 +4394,6 @@
     <mergeCell ref="D70:H70"/>
     <mergeCell ref="D71:H71"/>
     <mergeCell ref="D72:H72"/>
-    <mergeCell ref="D90:H90"/>
-    <mergeCell ref="D91:H91"/>
-    <mergeCell ref="D86:H86"/>
-    <mergeCell ref="D75:H75"/>
-    <mergeCell ref="D76:H76"/>
-    <mergeCell ref="D77:H77"/>
-    <mergeCell ref="D78:H78"/>
-    <mergeCell ref="D79:H79"/>
-    <mergeCell ref="D80:H80"/>
-    <mergeCell ref="D81:H81"/>
-    <mergeCell ref="D82:H82"/>
-    <mergeCell ref="D83:H83"/>
-    <mergeCell ref="D84:H84"/>
-    <mergeCell ref="D85:H85"/>
-    <mergeCell ref="D73:H73"/>
-    <mergeCell ref="D62:H62"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D56:H56"/>
-    <mergeCell ref="D57:H57"/>
-    <mergeCell ref="D58:H58"/>
-    <mergeCell ref="D59:H59"/>
-    <mergeCell ref="D60:H60"/>
-    <mergeCell ref="D61:H61"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4435,13 +4435,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -4495,13 +4495,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -4693,13 +4693,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="42" t="s">
+      <c r="D22" s="43" t="s">
         <v>387</v>
       </c>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="45"/>
     </row>
     <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -4967,16 +4967,24 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D22:H22"/>
@@ -4989,24 +4997,16 @@
     <mergeCell ref="D29:H29"/>
     <mergeCell ref="D30:H30"/>
     <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5283,14 +5283,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="D2:H2"/>
@@ -5303,6 +5295,14 @@
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5344,13 +5344,13 @@
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="45" t="s">
+      <c r="D8" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="45"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -5404,13 +5404,13 @@
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="36" t="s">
+      <c r="D13" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="38"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="42"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -5758,13 +5758,13 @@
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="42" t="s">
+      <c r="D40" s="43" t="s">
         <v>308</v>
       </c>
-      <c r="E40" s="43"/>
-      <c r="F40" s="43"/>
-      <c r="G40" s="43"/>
-      <c r="H40" s="44"/>
+      <c r="E40" s="44"/>
+      <c r="F40" s="44"/>
+      <c r="G40" s="44"/>
+      <c r="H40" s="45"/>
     </row>
     <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -5878,13 +5878,13 @@
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
-      <c r="D49" s="39" t="s">
+      <c r="D49" s="36" t="s">
         <v>253</v>
       </c>
-      <c r="E49" s="40"/>
-      <c r="F49" s="40"/>
-      <c r="G49" s="40"/>
-      <c r="H49" s="41"/>
+      <c r="E49" s="37"/>
+      <c r="F49" s="37"/>
+      <c r="G49" s="37"/>
+      <c r="H49" s="38"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
@@ -5902,25 +5902,25 @@
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="39" t="s">
+      <c r="D51" s="36" t="s">
         <v>254</v>
       </c>
-      <c r="E51" s="40"/>
-      <c r="F51" s="40"/>
-      <c r="G51" s="40"/>
-      <c r="H51" s="41"/>
+      <c r="E51" s="37"/>
+      <c r="F51" s="37"/>
+      <c r="G51" s="37"/>
+      <c r="H51" s="38"/>
     </row>
     <row r="52" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="39" t="s">
+      <c r="D52" s="36" t="s">
         <v>311</v>
       </c>
-      <c r="E52" s="40"/>
-      <c r="F52" s="40"/>
-      <c r="G52" s="40"/>
-      <c r="H52" s="41"/>
+      <c r="E52" s="37"/>
+      <c r="F52" s="37"/>
+      <c r="G52" s="37"/>
+      <c r="H52" s="38"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
@@ -6044,36 +6044,12 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D59:H59"/>
-    <mergeCell ref="D60:H60"/>
-    <mergeCell ref="D61:H61"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D58:H58"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D56:H56"/>
-    <mergeCell ref="D57:H57"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D34:H34"/>
@@ -6090,12 +6066,36 @@
     <mergeCell ref="D30:H30"/>
     <mergeCell ref="D31:H31"/>
     <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D57:H57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6142,13 +6142,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6166,49 +6166,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="38"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="42"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="36" t="s">
+      <c r="D5" s="40" t="s">
         <v>313</v>
       </c>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="42"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="36" t="s">
+      <c r="D6" s="40" t="s">
         <v>314</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="38"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="42"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -6388,13 +6388,13 @@
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="39" t="s">
+      <c r="D21" s="36" t="s">
         <v>319</v>
       </c>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="41"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="38"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -6572,15 +6572,18 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
     <mergeCell ref="D25:H25"/>
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="D15:H15"/>
@@ -6593,18 +6596,15 @@
     <mergeCell ref="D22:H22"/>
     <mergeCell ref="D23:H23"/>
     <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
   </mergeCells>
   <pageMargins left="0.70866141732283461" right="0.70866141732283461" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6647,13 +6647,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6707,13 +6707,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
@@ -6917,13 +6917,13 @@
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="42" t="s">
+      <c r="D23" s="43" t="s">
         <v>297</v>
       </c>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="45"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
@@ -7025,13 +7025,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="39" t="s">
+      <c r="D31" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="41"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="38"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -7049,25 +7049,25 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="39" t="s">
+      <c r="D33" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="E33" s="40"/>
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="41"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="38"/>
     </row>
     <row r="34" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="39" t="s">
+      <c r="D34" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="E34" s="40"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="41"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="38"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -7191,16 +7191,24 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D22:H22"/>
     <mergeCell ref="D23:H23"/>
@@ -7213,24 +7221,16 @@
     <mergeCell ref="D30:H30"/>
     <mergeCell ref="D31:H31"/>
     <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7273,13 +7273,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -7333,13 +7333,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -7531,61 +7531,61 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="42" t="s">
+      <c r="D22" s="43" t="s">
         <v>272</v>
       </c>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="45"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="42" t="s">
+      <c r="D23" s="43" t="s">
         <v>326</v>
       </c>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="45"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
-      <c r="D24" s="42" t="s">
+      <c r="D24" s="43" t="s">
         <v>327</v>
       </c>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="45"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="42" t="s">
+      <c r="D25" s="43" t="s">
         <v>328</v>
       </c>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="45"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-      <c r="D26" s="42" t="s">
+      <c r="D26" s="43" t="s">
         <v>329</v>
       </c>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="44"/>
+      <c r="E26" s="44"/>
+      <c r="F26" s="44"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="45"/>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
@@ -7687,13 +7687,13 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="39" t="s">
+      <c r="D34" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="E34" s="40"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="41"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="38"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -7711,25 +7711,25 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
-      <c r="D36" s="39" t="s">
+      <c r="D36" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="E36" s="40"/>
-      <c r="F36" s="40"/>
-      <c r="G36" s="40"/>
-      <c r="H36" s="41"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="37"/>
+      <c r="G36" s="37"/>
+      <c r="H36" s="38"/>
     </row>
     <row r="37" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="39" t="s">
+      <c r="D37" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="E37" s="40"/>
-      <c r="F37" s="40"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="41"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
+      <c r="G37" s="37"/>
+      <c r="H37" s="38"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -7853,6 +7853,34 @@
     </row>
   </sheetData>
   <mergeCells count="44">
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
     <mergeCell ref="D35:H35"/>
     <mergeCell ref="D36:H36"/>
     <mergeCell ref="D21:H21"/>
@@ -7869,34 +7897,6 @@
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7939,13 +7939,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -7999,13 +7999,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8287,13 +8287,13 @@
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-      <c r="D29" s="42" t="s">
+      <c r="D29" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="43"/>
-      <c r="H29" s="44"/>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="44"/>
+      <c r="H29" s="45"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -8323,13 +8323,13 @@
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="46" t="s">
+      <c r="D32" s="49" t="s">
         <v>337</v>
       </c>
-      <c r="E32" s="47"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="47"/>
-      <c r="H32" s="48"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="50"/>
+      <c r="G32" s="50"/>
+      <c r="H32" s="51"/>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
@@ -8349,25 +8349,25 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="49" t="s">
+      <c r="D34" s="52" t="s">
         <v>338</v>
       </c>
-      <c r="E34" s="50"/>
-      <c r="F34" s="50"/>
-      <c r="G34" s="50"/>
-      <c r="H34" s="51"/>
+      <c r="E34" s="53"/>
+      <c r="F34" s="53"/>
+      <c r="G34" s="53"/>
+      <c r="H34" s="54"/>
     </row>
     <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
-      <c r="D35" s="52" t="s">
+      <c r="D35" s="55" t="s">
         <v>340</v>
       </c>
-      <c r="E35" s="53"/>
-      <c r="F35" s="53"/>
-      <c r="G35" s="53"/>
-      <c r="H35" s="54"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="56"/>
+      <c r="G35" s="56"/>
+      <c r="H35" s="57"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -8391,13 +8391,13 @@
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="39" t="s">
+      <c r="D37" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="E37" s="40"/>
-      <c r="F37" s="40"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="41"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
+      <c r="G37" s="37"/>
+      <c r="H37" s="38"/>
     </row>
     <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
@@ -8457,13 +8457,13 @@
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="39" t="s">
+      <c r="D42" s="36" t="s">
         <v>274</v>
       </c>
-      <c r="E42" s="40"/>
-      <c r="F42" s="40"/>
-      <c r="G42" s="40"/>
-      <c r="H42" s="41"/>
+      <c r="E42" s="37"/>
+      <c r="F42" s="37"/>
+      <c r="G42" s="37"/>
+      <c r="H42" s="38"/>
     </row>
     <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
@@ -8481,25 +8481,25 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="39" t="s">
+      <c r="D44" s="36" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="40"/>
-      <c r="F44" s="40"/>
-      <c r="G44" s="40"/>
-      <c r="H44" s="41"/>
+      <c r="E44" s="37"/>
+      <c r="F44" s="37"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="38"/>
     </row>
     <row r="45" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
-      <c r="D45" s="39" t="s">
+      <c r="D45" s="36" t="s">
         <v>276</v>
       </c>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="41"/>
+      <c r="E45" s="37"/>
+      <c r="F45" s="37"/>
+      <c r="G45" s="37"/>
+      <c r="H45" s="38"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
@@ -8523,25 +8523,25 @@
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="39" t="s">
+      <c r="D47" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="E47" s="40"/>
-      <c r="F47" s="40"/>
-      <c r="G47" s="40"/>
-      <c r="H47" s="41"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="37"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="38"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="D48" s="39" t="s">
+      <c r="D48" s="36" t="s">
         <v>146</v>
       </c>
-      <c r="E48" s="40"/>
-      <c r="F48" s="40"/>
-      <c r="G48" s="40"/>
-      <c r="H48" s="41"/>
+      <c r="E48" s="37"/>
+      <c r="F48" s="37"/>
+      <c r="G48" s="37"/>
+      <c r="H48" s="38"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -8553,61 +8553,61 @@
       <c r="C49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D49" s="55" t="s">
+      <c r="D49" s="46" t="s">
         <v>278</v>
       </c>
-      <c r="E49" s="56"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="56"/>
-      <c r="H49" s="57"/>
+      <c r="E49" s="47"/>
+      <c r="F49" s="47"/>
+      <c r="G49" s="47"/>
+      <c r="H49" s="48"/>
     </row>
     <row r="50" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="D50" s="39" t="s">
+      <c r="D50" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="E50" s="40"/>
-      <c r="F50" s="40"/>
-      <c r="G50" s="40"/>
-      <c r="H50" s="41"/>
+      <c r="E50" s="37"/>
+      <c r="F50" s="37"/>
+      <c r="G50" s="37"/>
+      <c r="H50" s="38"/>
     </row>
     <row r="51" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="39" t="s">
+      <c r="D51" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="E51" s="40"/>
-      <c r="F51" s="40"/>
-      <c r="G51" s="40"/>
-      <c r="H51" s="41"/>
+      <c r="E51" s="37"/>
+      <c r="F51" s="37"/>
+      <c r="G51" s="37"/>
+      <c r="H51" s="38"/>
     </row>
     <row r="52" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="39" t="s">
+      <c r="D52" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="E52" s="40"/>
-      <c r="F52" s="40"/>
-      <c r="G52" s="40"/>
-      <c r="H52" s="41"/>
+      <c r="E52" s="37"/>
+      <c r="F52" s="37"/>
+      <c r="G52" s="37"/>
+      <c r="H52" s="38"/>
     </row>
     <row r="53" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
-      <c r="D53" s="39" t="s">
+      <c r="D53" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="E53" s="40"/>
-      <c r="F53" s="40"/>
-      <c r="G53" s="40"/>
-      <c r="H53" s="41"/>
+      <c r="E53" s="37"/>
+      <c r="F53" s="37"/>
+      <c r="G53" s="37"/>
+      <c r="H53" s="38"/>
     </row>
     <row r="54" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
@@ -8623,39 +8623,6 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D8:H8"/>
@@ -8672,6 +8639,39 @@
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="D22:H22"/>
     <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D49:H49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -8714,13 +8714,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -8774,13 +8774,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8972,13 +8972,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="42" t="s">
+      <c r="D22" s="43" t="s">
         <v>349</v>
       </c>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="45"/>
     </row>
     <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -9258,15 +9258,24 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
     <mergeCell ref="D34:H34"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D22:H22"/>
@@ -9281,24 +9290,15 @@
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9339,13 +9339,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -9399,13 +9399,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -9813,25 +9813,25 @@
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="39" t="s">
+      <c r="D39" s="36" t="s">
         <v>356</v>
       </c>
-      <c r="E39" s="40"/>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="41"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="37"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="38"/>
     </row>
     <row r="40" spans="1:8" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="39" t="s">
+      <c r="D40" s="36" t="s">
         <v>357</v>
       </c>
-      <c r="E40" s="40"/>
-      <c r="F40" s="40"/>
-      <c r="G40" s="40"/>
-      <c r="H40" s="41"/>
+      <c r="E40" s="37"/>
+      <c r="F40" s="37"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="38"/>
     </row>
     <row r="41" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -10008,6 +10008,41 @@
     </row>
   </sheetData>
   <mergeCells count="51">
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
     <mergeCell ref="D53:H53"/>
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="D22:H22"/>
@@ -10024,41 +10059,6 @@
     <mergeCell ref="D24:H24"/>
     <mergeCell ref="D25:H25"/>
     <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -10122,13 +10122,13 @@
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="40" t="s">
         <v>205</v>
       </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="38"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="42"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -10380,13 +10380,13 @@
       <c r="A24" s="12"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="42" t="s">
+      <c r="D24" s="43" t="s">
         <v>206</v>
       </c>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="45"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="12"/>
@@ -10786,16 +10786,36 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
     <mergeCell ref="D45:H45"/>
     <mergeCell ref="D34:H34"/>
     <mergeCell ref="D35:H35"/>
@@ -10808,36 +10828,16 @@
     <mergeCell ref="D42:H42"/>
     <mergeCell ref="D43:H43"/>
     <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Ampliando las fotos del pdf
</commit_message>
<xml_diff>
--- a/apiService/Plantilla-modelo.xlsx
+++ b/apiService/Plantilla-modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollo-software\reporte-obras-main\apiService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BE6827-62F7-408F-993E-FDBF619E2ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32292B18-3D95-4F97-B2CE-40D53F1751A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="947" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1443,7 +1443,7 @@
     <t xml:space="preserve">2.2  Comprobar bomba grupo presión 2:          </t>
   </si>
   <si>
-    <t>4.5 Verificar seguridades (FOTOS del cuadro antes y después) prueba nueva 2</t>
+    <t>4.5 Verificar seguridades (FOTOS del cuadro antes y después) prueba nueva 3</t>
   </si>
 </sst>
 </file>
@@ -1684,6 +1684,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1693,12 +1696,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1708,14 +1705,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1743,6 +1734,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -2122,13 +2122,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -2158,13 +2158,13 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -2454,13 +2454,13 @@
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="43" t="s">
+      <c r="D27" s="42" t="s">
         <v>162</v>
       </c>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="45"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="44"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
@@ -2532,25 +2532,25 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="40" t="s">
+      <c r="D33" s="36" t="s">
         <v>156</v>
       </c>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="42"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="38"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="14"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="36" t="s">
+      <c r="D34" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="E34" s="37"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="37"/>
-      <c r="H34" s="38"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="41"/>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -2610,13 +2610,13 @@
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="36" t="s">
+      <c r="D39" s="39" t="s">
         <v>241</v>
       </c>
-      <c r="E39" s="37"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="37"/>
-      <c r="H39" s="38"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="40"/>
+      <c r="H39" s="41"/>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -2769,6 +2769,32 @@
     <row r="282" ht="45" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D16:H16"/>
@@ -2785,32 +2811,6 @@
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D43:H43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3082,13 +3082,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="D4:H4"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D8:H8"/>
@@ -3101,6 +3094,13 @@
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="D4:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3143,13 +3143,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -3167,49 +3167,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="42"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="36" t="s">
         <v>365</v>
       </c>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="42"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="38"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -3401,85 +3401,85 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="36" t="s">
+      <c r="D22" s="39" t="s">
         <v>371</v>
       </c>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="41"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="36" t="s">
+      <c r="D23" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="37"/>
-      <c r="H23" s="38"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="41"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="36" t="s">
+      <c r="D24" s="39" t="s">
         <v>374</v>
       </c>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="41"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="36" t="s">
+      <c r="D25" s="39" t="s">
         <v>375</v>
       </c>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="38"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="41"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="36" t="s">
+      <c r="D26" s="39" t="s">
         <v>373</v>
       </c>
-      <c r="E26" s="37"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="38"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="41"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="12"/>
-      <c r="D27" s="36" t="s">
+      <c r="D27" s="39" t="s">
         <v>372</v>
       </c>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="38"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="41"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="12"/>
-      <c r="D28" s="36" t="s">
+      <c r="D28" s="39" t="s">
         <v>231</v>
       </c>
-      <c r="E28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="38"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="41"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3515,13 +3515,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="36" t="s">
+      <c r="D31" s="39" t="s">
         <v>376</v>
       </c>
-      <c r="E31" s="37"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="38"/>
+      <c r="E31" s="40"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="41"/>
     </row>
     <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -3689,13 +3689,13 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="40" t="s">
+      <c r="D44" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="E44" s="41"/>
-      <c r="F44" s="41"/>
-      <c r="G44" s="41"/>
-      <c r="H44" s="42"/>
+      <c r="E44" s="37"/>
+      <c r="F44" s="37"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="38"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
@@ -3713,25 +3713,25 @@
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
-      <c r="D46" s="40" t="s">
+      <c r="D46" s="36" t="s">
         <v>378</v>
       </c>
-      <c r="E46" s="41"/>
-      <c r="F46" s="41"/>
-      <c r="G46" s="41"/>
-      <c r="H46" s="42"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="38"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="40" t="s">
+      <c r="D47" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="E47" s="41"/>
-      <c r="F47" s="41"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="42"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="37"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="38"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3875,13 +3875,13 @@
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
-      <c r="D58" s="43" t="s">
+      <c r="D58" s="42" t="s">
         <v>114</v>
       </c>
-      <c r="E58" s="44"/>
-      <c r="F58" s="44"/>
-      <c r="G58" s="44"/>
-      <c r="H58" s="45"/>
+      <c r="E58" s="43"/>
+      <c r="F58" s="43"/>
+      <c r="G58" s="43"/>
+      <c r="H58" s="44"/>
     </row>
     <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
@@ -4305,24 +4305,61 @@
     </row>
   </sheetData>
   <mergeCells count="89">
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D87:H87"/>
+    <mergeCell ref="D88:H88"/>
+    <mergeCell ref="D89:H89"/>
+    <mergeCell ref="D74:H74"/>
+    <mergeCell ref="D63:H63"/>
+    <mergeCell ref="D64:H64"/>
+    <mergeCell ref="D65:H65"/>
+    <mergeCell ref="D66:H66"/>
+    <mergeCell ref="D67:H67"/>
+    <mergeCell ref="D68:H68"/>
+    <mergeCell ref="D69:H69"/>
+    <mergeCell ref="D70:H70"/>
+    <mergeCell ref="D71:H71"/>
+    <mergeCell ref="D72:H72"/>
+    <mergeCell ref="D90:H90"/>
+    <mergeCell ref="D91:H91"/>
+    <mergeCell ref="D86:H86"/>
+    <mergeCell ref="D75:H75"/>
+    <mergeCell ref="D76:H76"/>
+    <mergeCell ref="D77:H77"/>
+    <mergeCell ref="D78:H78"/>
+    <mergeCell ref="D79:H79"/>
+    <mergeCell ref="D80:H80"/>
+    <mergeCell ref="D81:H81"/>
+    <mergeCell ref="D82:H82"/>
+    <mergeCell ref="D83:H83"/>
+    <mergeCell ref="D84:H84"/>
+    <mergeCell ref="D85:H85"/>
+    <mergeCell ref="D73:H73"/>
+    <mergeCell ref="D62:H62"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
     <mergeCell ref="D37:H37"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D21:H21"/>
@@ -4339,61 +4376,24 @@
     <mergeCell ref="D25:H25"/>
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D73:H73"/>
-    <mergeCell ref="D62:H62"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D56:H56"/>
-    <mergeCell ref="D57:H57"/>
-    <mergeCell ref="D58:H58"/>
-    <mergeCell ref="D59:H59"/>
-    <mergeCell ref="D60:H60"/>
-    <mergeCell ref="D61:H61"/>
-    <mergeCell ref="D90:H90"/>
-    <mergeCell ref="D91:H91"/>
-    <mergeCell ref="D86:H86"/>
-    <mergeCell ref="D75:H75"/>
-    <mergeCell ref="D76:H76"/>
-    <mergeCell ref="D77:H77"/>
-    <mergeCell ref="D78:H78"/>
-    <mergeCell ref="D79:H79"/>
-    <mergeCell ref="D80:H80"/>
-    <mergeCell ref="D81:H81"/>
-    <mergeCell ref="D82:H82"/>
-    <mergeCell ref="D83:H83"/>
-    <mergeCell ref="D84:H84"/>
-    <mergeCell ref="D85:H85"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D87:H87"/>
-    <mergeCell ref="D88:H88"/>
-    <mergeCell ref="D89:H89"/>
-    <mergeCell ref="D74:H74"/>
-    <mergeCell ref="D63:H63"/>
-    <mergeCell ref="D64:H64"/>
-    <mergeCell ref="D65:H65"/>
-    <mergeCell ref="D66:H66"/>
-    <mergeCell ref="D67:H67"/>
-    <mergeCell ref="D68:H68"/>
-    <mergeCell ref="D69:H69"/>
-    <mergeCell ref="D70:H70"/>
-    <mergeCell ref="D71:H71"/>
-    <mergeCell ref="D72:H72"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4435,13 +4435,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -4495,13 +4495,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -4693,13 +4693,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="42" t="s">
         <v>387</v>
       </c>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="45"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="44"/>
     </row>
     <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -4967,12 +4967,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
@@ -4985,28 +5001,12 @@
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5283,6 +5283,14 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="D2:H2"/>
@@ -5295,14 +5303,6 @@
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5344,13 +5344,13 @@
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -5404,13 +5404,13 @@
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="38"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -5758,13 +5758,13 @@
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="43" t="s">
+      <c r="D40" s="42" t="s">
         <v>308</v>
       </c>
-      <c r="E40" s="44"/>
-      <c r="F40" s="44"/>
-      <c r="G40" s="44"/>
-      <c r="H40" s="45"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="44"/>
     </row>
     <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -5878,13 +5878,13 @@
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
-      <c r="D49" s="36" t="s">
+      <c r="D49" s="39" t="s">
         <v>253</v>
       </c>
-      <c r="E49" s="37"/>
-      <c r="F49" s="37"/>
-      <c r="G49" s="37"/>
-      <c r="H49" s="38"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
+      <c r="G49" s="40"/>
+      <c r="H49" s="41"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
@@ -5902,25 +5902,25 @@
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="36" t="s">
+      <c r="D51" s="39" t="s">
         <v>254</v>
       </c>
-      <c r="E51" s="37"/>
-      <c r="F51" s="37"/>
-      <c r="G51" s="37"/>
-      <c r="H51" s="38"/>
+      <c r="E51" s="40"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="41"/>
     </row>
     <row r="52" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="36" t="s">
+      <c r="D52" s="39" t="s">
         <v>311</v>
       </c>
-      <c r="E52" s="37"/>
-      <c r="F52" s="37"/>
-      <c r="G52" s="37"/>
-      <c r="H52" s="38"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="40"/>
+      <c r="G52" s="40"/>
+      <c r="H52" s="41"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
@@ -6044,12 +6044,36 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D34:H34"/>
@@ -6066,36 +6090,12 @@
     <mergeCell ref="D30:H30"/>
     <mergeCell ref="D31:H31"/>
     <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D59:H59"/>
-    <mergeCell ref="D60:H60"/>
-    <mergeCell ref="D61:H61"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D58:H58"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D56:H56"/>
-    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6142,13 +6142,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6166,49 +6166,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="42"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="36" t="s">
         <v>313</v>
       </c>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="36" t="s">
         <v>314</v>
       </c>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="42"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="38"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -6388,13 +6388,13 @@
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="36" t="s">
+      <c r="D21" s="39" t="s">
         <v>319</v>
       </c>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="38"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="41"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -6572,6 +6572,27 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="D2:H2"/>
@@ -6584,27 +6605,6 @@
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
     <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
   </mergeCells>
   <pageMargins left="0.70866141732283461" right="0.70866141732283461" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6647,13 +6647,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6707,13 +6707,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
@@ -6917,13 +6917,13 @@
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="42" t="s">
         <v>297</v>
       </c>
-      <c r="E23" s="44"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="45"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="44"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
@@ -7025,13 +7025,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="36" t="s">
+      <c r="D31" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="37"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="38"/>
+      <c r="E31" s="40"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="41"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -7049,25 +7049,25 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="36" t="s">
+      <c r="D33" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="37"/>
-      <c r="H33" s="38"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="40"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="41"/>
     </row>
     <row r="34" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="36" t="s">
+      <c r="D34" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="E34" s="37"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="37"/>
-      <c r="H34" s="38"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="41"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -7191,12 +7191,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
@@ -7209,28 +7225,12 @@
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7273,13 +7273,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -7333,13 +7333,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -7531,61 +7531,61 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="42" t="s">
         <v>272</v>
       </c>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="45"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="44"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="42" t="s">
         <v>326</v>
       </c>
-      <c r="E23" s="44"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="45"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="44"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="42" t="s">
         <v>327</v>
       </c>
-      <c r="E24" s="44"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="45"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="43"/>
+      <c r="H24" s="44"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="42" t="s">
         <v>328</v>
       </c>
-      <c r="E25" s="44"/>
-      <c r="F25" s="44"/>
-      <c r="G25" s="44"/>
-      <c r="H25" s="45"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="43"/>
+      <c r="H25" s="44"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-      <c r="D26" s="43" t="s">
+      <c r="D26" s="42" t="s">
         <v>329</v>
       </c>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="45"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="43"/>
+      <c r="H26" s="44"/>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
@@ -7687,13 +7687,13 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="36" t="s">
+      <c r="D34" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E34" s="37"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="37"/>
-      <c r="H34" s="38"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="41"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -7711,25 +7711,25 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
-      <c r="D36" s="36" t="s">
+      <c r="D36" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="E36" s="37"/>
-      <c r="F36" s="37"/>
-      <c r="G36" s="37"/>
-      <c r="H36" s="38"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="40"/>
+      <c r="G36" s="40"/>
+      <c r="H36" s="41"/>
     </row>
     <row r="37" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="36" t="s">
+      <c r="D37" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="38"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="40"/>
+      <c r="G37" s="40"/>
+      <c r="H37" s="41"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -7853,34 +7853,6 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
     <mergeCell ref="D35:H35"/>
     <mergeCell ref="D36:H36"/>
     <mergeCell ref="D21:H21"/>
@@ -7897,6 +7869,34 @@
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7939,13 +7939,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -7999,13 +7999,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8287,13 +8287,13 @@
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-      <c r="D29" s="43" t="s">
+      <c r="D29" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="45"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="43"/>
+      <c r="G29" s="43"/>
+      <c r="H29" s="44"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -8323,13 +8323,13 @@
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="49" t="s">
+      <c r="D32" s="46" t="s">
         <v>337</v>
       </c>
-      <c r="E32" s="50"/>
-      <c r="F32" s="50"/>
-      <c r="G32" s="50"/>
-      <c r="H32" s="51"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="47"/>
+      <c r="G32" s="47"/>
+      <c r="H32" s="48"/>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
@@ -8349,25 +8349,25 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="52" t="s">
+      <c r="D34" s="49" t="s">
         <v>338</v>
       </c>
-      <c r="E34" s="53"/>
-      <c r="F34" s="53"/>
-      <c r="G34" s="53"/>
-      <c r="H34" s="54"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="50"/>
+      <c r="G34" s="50"/>
+      <c r="H34" s="51"/>
     </row>
     <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
-      <c r="D35" s="55" t="s">
+      <c r="D35" s="52" t="s">
         <v>340</v>
       </c>
-      <c r="E35" s="56"/>
-      <c r="F35" s="56"/>
-      <c r="G35" s="56"/>
-      <c r="H35" s="57"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="54"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -8391,13 +8391,13 @@
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="36" t="s">
+      <c r="D37" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="38"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="40"/>
+      <c r="G37" s="40"/>
+      <c r="H37" s="41"/>
     </row>
     <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
@@ -8457,13 +8457,13 @@
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="36" t="s">
+      <c r="D42" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="E42" s="37"/>
-      <c r="F42" s="37"/>
-      <c r="G42" s="37"/>
-      <c r="H42" s="38"/>
+      <c r="E42" s="40"/>
+      <c r="F42" s="40"/>
+      <c r="G42" s="40"/>
+      <c r="H42" s="41"/>
     </row>
     <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
@@ -8481,25 +8481,25 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="36" t="s">
+      <c r="D44" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="37"/>
-      <c r="F44" s="37"/>
-      <c r="G44" s="37"/>
-      <c r="H44" s="38"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40"/>
+      <c r="G44" s="40"/>
+      <c r="H44" s="41"/>
     </row>
     <row r="45" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
-      <c r="D45" s="36" t="s">
+      <c r="D45" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="E45" s="37"/>
-      <c r="F45" s="37"/>
-      <c r="G45" s="37"/>
-      <c r="H45" s="38"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="41"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
@@ -8523,25 +8523,25 @@
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="36" t="s">
+      <c r="D47" s="39" t="s">
         <v>145</v>
       </c>
-      <c r="E47" s="37"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="37"/>
-      <c r="H47" s="38"/>
+      <c r="E47" s="40"/>
+      <c r="F47" s="40"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="41"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="D48" s="36" t="s">
+      <c r="D48" s="39" t="s">
         <v>146</v>
       </c>
-      <c r="E48" s="37"/>
-      <c r="F48" s="37"/>
-      <c r="G48" s="37"/>
-      <c r="H48" s="38"/>
+      <c r="E48" s="40"/>
+      <c r="F48" s="40"/>
+      <c r="G48" s="40"/>
+      <c r="H48" s="41"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -8553,61 +8553,61 @@
       <c r="C49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D49" s="46" t="s">
+      <c r="D49" s="55" t="s">
         <v>278</v>
       </c>
-      <c r="E49" s="47"/>
-      <c r="F49" s="47"/>
-      <c r="G49" s="47"/>
-      <c r="H49" s="48"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="57"/>
     </row>
     <row r="50" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="D50" s="36" t="s">
+      <c r="D50" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="E50" s="37"/>
-      <c r="F50" s="37"/>
-      <c r="G50" s="37"/>
-      <c r="H50" s="38"/>
+      <c r="E50" s="40"/>
+      <c r="F50" s="40"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="41"/>
     </row>
     <row r="51" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="36" t="s">
+      <c r="D51" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="E51" s="37"/>
-      <c r="F51" s="37"/>
-      <c r="G51" s="37"/>
-      <c r="H51" s="38"/>
+      <c r="E51" s="40"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="41"/>
     </row>
     <row r="52" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="36" t="s">
+      <c r="D52" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="E52" s="37"/>
-      <c r="F52" s="37"/>
-      <c r="G52" s="37"/>
-      <c r="H52" s="38"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="40"/>
+      <c r="G52" s="40"/>
+      <c r="H52" s="41"/>
     </row>
     <row r="53" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
-      <c r="D53" s="36" t="s">
+      <c r="D53" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="E53" s="37"/>
-      <c r="F53" s="37"/>
-      <c r="G53" s="37"/>
-      <c r="H53" s="38"/>
+      <c r="E53" s="40"/>
+      <c r="F53" s="40"/>
+      <c r="G53" s="40"/>
+      <c r="H53" s="41"/>
     </row>
     <row r="54" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
@@ -8623,6 +8623,39 @@
     </row>
   </sheetData>
   <mergeCells count="49">
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D8:H8"/>
@@ -8639,39 +8672,6 @@
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="D22:H22"/>
     <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D49:H49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -8714,13 +8714,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -8774,13 +8774,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8972,13 +8972,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="42" t="s">
         <v>349</v>
       </c>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="45"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="44"/>
     </row>
     <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -9258,24 +9258,15 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
     <mergeCell ref="D34:H34"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D22:H22"/>
@@ -9290,15 +9281,24 @@
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9339,13 +9339,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -9399,13 +9399,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -9813,25 +9813,25 @@
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="36" t="s">
+      <c r="D39" s="39" t="s">
         <v>356</v>
       </c>
-      <c r="E39" s="37"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="37"/>
-      <c r="H39" s="38"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="40"/>
+      <c r="H39" s="41"/>
     </row>
     <row r="40" spans="1:8" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="36" t="s">
+      <c r="D40" s="39" t="s">
         <v>357</v>
       </c>
-      <c r="E40" s="37"/>
-      <c r="F40" s="37"/>
-      <c r="G40" s="37"/>
-      <c r="H40" s="38"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="40"/>
+      <c r="H40" s="41"/>
     </row>
     <row r="41" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -10008,25 +10008,22 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D36:H36"/>
     <mergeCell ref="D31:H31"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D52:H52"/>
@@ -10043,22 +10040,25 @@
     <mergeCell ref="D45:H45"/>
     <mergeCell ref="D46:H46"/>
     <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -10122,13 +10122,13 @@
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="36" t="s">
         <v>205</v>
       </c>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="42"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -10380,13 +10380,13 @@
       <c r="A24" s="12"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="42" t="s">
         <v>206</v>
       </c>
-      <c r="E24" s="44"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="45"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="43"/>
+      <c r="H24" s="44"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="12"/>
@@ -10786,12 +10786,40 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D8:H8"/>
     <mergeCell ref="D9:H9"/>
@@ -10804,40 +10832,12 @@
     <mergeCell ref="D16:H16"/>
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Probando sincronizacion de excel
</commit_message>
<xml_diff>
--- a/apiService/Plantilla-modelo.xlsx
+++ b/apiService/Plantilla-modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollo-software\reporte-obras-main\apiService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FEDF456-D617-4968-BB64-4089A641AD7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD26FECF-F63F-4796-9765-22EC35C8E990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="947" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="392">
   <si>
     <t>REVISADO</t>
   </si>
@@ -1441,9 +1441,6 @@
   </si>
   <si>
     <t xml:space="preserve">2.2  Comprobar bomba grupo presión 2:          </t>
-  </si>
-  <si>
-    <t>4.5 Verificar seguridades (FOTOS del cuadro antes y después) prueba nueva 3</t>
   </si>
 </sst>
 </file>
@@ -1593,7 +1590,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1684,6 +1681,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1693,12 +1693,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1708,14 +1702,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1744,16 +1732,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2131,13 +2119,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -2167,13 +2155,13 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -2463,13 +2451,13 @@
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="43" t="s">
+      <c r="D27" s="42" t="s">
         <v>162</v>
       </c>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="45"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="44"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
@@ -2541,25 +2529,25 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="40" t="s">
+      <c r="D33" s="36" t="s">
         <v>156</v>
       </c>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="42"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="38"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="14"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="36" t="s">
+      <c r="D34" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="E34" s="37"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="37"/>
-      <c r="H34" s="38"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="41"/>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -2619,13 +2607,13 @@
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="36" t="s">
+      <c r="D39" s="39" t="s">
         <v>241</v>
       </c>
-      <c r="E39" s="37"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="37"/>
-      <c r="H39" s="38"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="40"/>
+      <c r="H39" s="41"/>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -2778,6 +2766,32 @@
     <row r="282" ht="45" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D16:H16"/>
@@ -2794,32 +2808,6 @@
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D43:H43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3091,13 +3079,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="D4:H4"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D8:H8"/>
@@ -3110,6 +3091,13 @@
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="D4:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3152,13 +3140,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -3176,49 +3164,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="42"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="36" t="s">
         <v>365</v>
       </c>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="42"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="38"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -3410,85 +3398,85 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="36" t="s">
+      <c r="D22" s="39" t="s">
         <v>371</v>
       </c>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="41"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="36" t="s">
+      <c r="D23" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="37"/>
-      <c r="H23" s="38"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="41"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="36" t="s">
+      <c r="D24" s="39" t="s">
         <v>374</v>
       </c>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="41"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="36" t="s">
+      <c r="D25" s="39" t="s">
         <v>375</v>
       </c>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="38"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="41"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="36" t="s">
+      <c r="D26" s="39" t="s">
         <v>373</v>
       </c>
-      <c r="E26" s="37"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="38"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="41"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="12"/>
-      <c r="D27" s="36" t="s">
+      <c r="D27" s="39" t="s">
         <v>372</v>
       </c>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="38"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="41"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="12"/>
-      <c r="D28" s="36" t="s">
+      <c r="D28" s="39" t="s">
         <v>231</v>
       </c>
-      <c r="E28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="38"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="41"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3524,13 +3512,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="36" t="s">
+      <c r="D31" s="39" t="s">
         <v>376</v>
       </c>
-      <c r="E31" s="37"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="38"/>
+      <c r="E31" s="40"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="41"/>
     </row>
     <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -3698,13 +3686,13 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="40" t="s">
+      <c r="D44" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="E44" s="41"/>
-      <c r="F44" s="41"/>
-      <c r="G44" s="41"/>
-      <c r="H44" s="42"/>
+      <c r="E44" s="37"/>
+      <c r="F44" s="37"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="38"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
@@ -3722,25 +3710,25 @@
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
-      <c r="D46" s="40" t="s">
+      <c r="D46" s="36" t="s">
         <v>378</v>
       </c>
-      <c r="E46" s="41"/>
-      <c r="F46" s="41"/>
-      <c r="G46" s="41"/>
-      <c r="H46" s="42"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="38"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="40" t="s">
+      <c r="D47" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="E47" s="41"/>
-      <c r="F47" s="41"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="42"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="37"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="38"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3884,13 +3872,13 @@
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
-      <c r="D58" s="43" t="s">
+      <c r="D58" s="42" t="s">
         <v>114</v>
       </c>
-      <c r="E58" s="44"/>
-      <c r="F58" s="44"/>
-      <c r="G58" s="44"/>
-      <c r="H58" s="45"/>
+      <c r="E58" s="43"/>
+      <c r="F58" s="43"/>
+      <c r="G58" s="43"/>
+      <c r="H58" s="44"/>
     </row>
     <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
@@ -4314,24 +4302,61 @@
     </row>
   </sheetData>
   <mergeCells count="89">
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D87:H87"/>
+    <mergeCell ref="D88:H88"/>
+    <mergeCell ref="D89:H89"/>
+    <mergeCell ref="D74:H74"/>
+    <mergeCell ref="D63:H63"/>
+    <mergeCell ref="D64:H64"/>
+    <mergeCell ref="D65:H65"/>
+    <mergeCell ref="D66:H66"/>
+    <mergeCell ref="D67:H67"/>
+    <mergeCell ref="D68:H68"/>
+    <mergeCell ref="D69:H69"/>
+    <mergeCell ref="D70:H70"/>
+    <mergeCell ref="D71:H71"/>
+    <mergeCell ref="D72:H72"/>
+    <mergeCell ref="D90:H90"/>
+    <mergeCell ref="D91:H91"/>
+    <mergeCell ref="D86:H86"/>
+    <mergeCell ref="D75:H75"/>
+    <mergeCell ref="D76:H76"/>
+    <mergeCell ref="D77:H77"/>
+    <mergeCell ref="D78:H78"/>
+    <mergeCell ref="D79:H79"/>
+    <mergeCell ref="D80:H80"/>
+    <mergeCell ref="D81:H81"/>
+    <mergeCell ref="D82:H82"/>
+    <mergeCell ref="D83:H83"/>
+    <mergeCell ref="D84:H84"/>
+    <mergeCell ref="D85:H85"/>
+    <mergeCell ref="D73:H73"/>
+    <mergeCell ref="D62:H62"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
     <mergeCell ref="D37:H37"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D21:H21"/>
@@ -4348,61 +4373,24 @@
     <mergeCell ref="D25:H25"/>
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D73:H73"/>
-    <mergeCell ref="D62:H62"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D56:H56"/>
-    <mergeCell ref="D57:H57"/>
-    <mergeCell ref="D58:H58"/>
-    <mergeCell ref="D59:H59"/>
-    <mergeCell ref="D60:H60"/>
-    <mergeCell ref="D61:H61"/>
-    <mergeCell ref="D90:H90"/>
-    <mergeCell ref="D91:H91"/>
-    <mergeCell ref="D86:H86"/>
-    <mergeCell ref="D75:H75"/>
-    <mergeCell ref="D76:H76"/>
-    <mergeCell ref="D77:H77"/>
-    <mergeCell ref="D78:H78"/>
-    <mergeCell ref="D79:H79"/>
-    <mergeCell ref="D80:H80"/>
-    <mergeCell ref="D81:H81"/>
-    <mergeCell ref="D82:H82"/>
-    <mergeCell ref="D83:H83"/>
-    <mergeCell ref="D84:H84"/>
-    <mergeCell ref="D85:H85"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D87:H87"/>
-    <mergeCell ref="D88:H88"/>
-    <mergeCell ref="D89:H89"/>
-    <mergeCell ref="D74:H74"/>
-    <mergeCell ref="D63:H63"/>
-    <mergeCell ref="D64:H64"/>
-    <mergeCell ref="D65:H65"/>
-    <mergeCell ref="D66:H66"/>
-    <mergeCell ref="D67:H67"/>
-    <mergeCell ref="D68:H68"/>
-    <mergeCell ref="D69:H69"/>
-    <mergeCell ref="D70:H70"/>
-    <mergeCell ref="D71:H71"/>
-    <mergeCell ref="D72:H72"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4444,13 +4432,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -4504,13 +4492,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -4702,13 +4690,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="42" t="s">
         <v>387</v>
       </c>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="45"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="44"/>
     </row>
     <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -4976,12 +4964,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
@@ -4994,28 +4998,12 @@
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5023,7 +5011,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6D5BD9-6748-4A03-A6F1-166697746BD8}">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -5278,20 +5266,15 @@
       <c r="G19" s="22"/>
       <c r="H19" s="23"/>
     </row>
-    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="59" t="s">
-        <v>392</v>
-      </c>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
-      <c r="H20" s="61"/>
-    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="19">
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="D2:H2"/>
@@ -5304,14 +5287,6 @@
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5353,13 +5328,13 @@
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -5413,13 +5388,13 @@
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="38"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -5767,13 +5742,13 @@
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="43" t="s">
+      <c r="D40" s="42" t="s">
         <v>308</v>
       </c>
-      <c r="E40" s="44"/>
-      <c r="F40" s="44"/>
-      <c r="G40" s="44"/>
-      <c r="H40" s="45"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="44"/>
     </row>
     <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -5887,13 +5862,13 @@
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
-      <c r="D49" s="36" t="s">
+      <c r="D49" s="39" t="s">
         <v>253</v>
       </c>
-      <c r="E49" s="37"/>
-      <c r="F49" s="37"/>
-      <c r="G49" s="37"/>
-      <c r="H49" s="38"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
+      <c r="G49" s="40"/>
+      <c r="H49" s="41"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
@@ -5911,25 +5886,25 @@
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="36" t="s">
+      <c r="D51" s="39" t="s">
         <v>254</v>
       </c>
-      <c r="E51" s="37"/>
-      <c r="F51" s="37"/>
-      <c r="G51" s="37"/>
-      <c r="H51" s="38"/>
+      <c r="E51" s="40"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="41"/>
     </row>
     <row r="52" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="36" t="s">
+      <c r="D52" s="39" t="s">
         <v>311</v>
       </c>
-      <c r="E52" s="37"/>
-      <c r="F52" s="37"/>
-      <c r="G52" s="37"/>
-      <c r="H52" s="38"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="40"/>
+      <c r="G52" s="40"/>
+      <c r="H52" s="41"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
@@ -6053,12 +6028,36 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D34:H34"/>
@@ -6075,36 +6074,12 @@
     <mergeCell ref="D30:H30"/>
     <mergeCell ref="D31:H31"/>
     <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D59:H59"/>
-    <mergeCell ref="D60:H60"/>
-    <mergeCell ref="D61:H61"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D58:H58"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D56:H56"/>
-    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6151,13 +6126,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6175,49 +6150,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="42"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="36" t="s">
         <v>313</v>
       </c>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="36" t="s">
         <v>314</v>
       </c>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="42"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="38"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -6397,13 +6372,13 @@
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="36" t="s">
+      <c r="D21" s="39" t="s">
         <v>319</v>
       </c>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="38"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="41"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -6581,6 +6556,27 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="D2:H2"/>
@@ -6593,27 +6589,6 @@
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
     <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
   </mergeCells>
   <pageMargins left="0.70866141732283461" right="0.70866141732283461" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6656,13 +6631,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6716,13 +6691,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
@@ -6926,13 +6901,13 @@
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="42" t="s">
         <v>297</v>
       </c>
-      <c r="E23" s="44"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="45"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="44"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
@@ -7034,13 +7009,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="36" t="s">
+      <c r="D31" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="37"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="38"/>
+      <c r="E31" s="40"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="41"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -7058,25 +7033,25 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="36" t="s">
+      <c r="D33" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="37"/>
-      <c r="H33" s="38"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="40"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="41"/>
     </row>
     <row r="34" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="36" t="s">
+      <c r="D34" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="E34" s="37"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="37"/>
-      <c r="H34" s="38"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="41"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -7200,12 +7175,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
@@ -7218,28 +7209,12 @@
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7282,13 +7257,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -7342,13 +7317,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -7540,61 +7515,61 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="42" t="s">
         <v>272</v>
       </c>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="45"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="44"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="42" t="s">
         <v>326</v>
       </c>
-      <c r="E23" s="44"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="45"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="44"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="42" t="s">
         <v>327</v>
       </c>
-      <c r="E24" s="44"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="45"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="43"/>
+      <c r="H24" s="44"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="42" t="s">
         <v>328</v>
       </c>
-      <c r="E25" s="44"/>
-      <c r="F25" s="44"/>
-      <c r="G25" s="44"/>
-      <c r="H25" s="45"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="43"/>
+      <c r="H25" s="44"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-      <c r="D26" s="43" t="s">
+      <c r="D26" s="42" t="s">
         <v>329</v>
       </c>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="45"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="43"/>
+      <c r="H26" s="44"/>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
@@ -7696,13 +7671,13 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="36" t="s">
+      <c r="D34" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E34" s="37"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="37"/>
-      <c r="H34" s="38"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="41"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -7720,25 +7695,25 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
-      <c r="D36" s="36" t="s">
+      <c r="D36" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="E36" s="37"/>
-      <c r="F36" s="37"/>
-      <c r="G36" s="37"/>
-      <c r="H36" s="38"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="40"/>
+      <c r="G36" s="40"/>
+      <c r="H36" s="41"/>
     </row>
     <row r="37" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="36" t="s">
+      <c r="D37" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="38"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="40"/>
+      <c r="G37" s="40"/>
+      <c r="H37" s="41"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -7862,34 +7837,6 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
     <mergeCell ref="D35:H35"/>
     <mergeCell ref="D36:H36"/>
     <mergeCell ref="D21:H21"/>
@@ -7906,6 +7853,34 @@
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7948,13 +7923,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -8008,13 +7983,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8296,13 +8271,13 @@
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-      <c r="D29" s="43" t="s">
+      <c r="D29" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="45"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="43"/>
+      <c r="G29" s="43"/>
+      <c r="H29" s="44"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -8332,13 +8307,13 @@
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="49" t="s">
+      <c r="D32" s="46" t="s">
         <v>337</v>
       </c>
-      <c r="E32" s="50"/>
-      <c r="F32" s="50"/>
-      <c r="G32" s="50"/>
-      <c r="H32" s="51"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="47"/>
+      <c r="G32" s="47"/>
+      <c r="H32" s="48"/>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
@@ -8358,25 +8333,25 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="52" t="s">
+      <c r="D34" s="49" t="s">
         <v>338</v>
       </c>
-      <c r="E34" s="53"/>
-      <c r="F34" s="53"/>
-      <c r="G34" s="53"/>
-      <c r="H34" s="54"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="50"/>
+      <c r="G34" s="50"/>
+      <c r="H34" s="51"/>
     </row>
     <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
-      <c r="D35" s="55" t="s">
+      <c r="D35" s="52" t="s">
         <v>340</v>
       </c>
-      <c r="E35" s="56"/>
-      <c r="F35" s="56"/>
-      <c r="G35" s="56"/>
-      <c r="H35" s="57"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="54"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -8400,13 +8375,13 @@
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="36" t="s">
+      <c r="D37" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="38"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="40"/>
+      <c r="G37" s="40"/>
+      <c r="H37" s="41"/>
     </row>
     <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
@@ -8466,13 +8441,13 @@
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="36" t="s">
+      <c r="D42" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="E42" s="37"/>
-      <c r="F42" s="37"/>
-      <c r="G42" s="37"/>
-      <c r="H42" s="38"/>
+      <c r="E42" s="40"/>
+      <c r="F42" s="40"/>
+      <c r="G42" s="40"/>
+      <c r="H42" s="41"/>
     </row>
     <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
@@ -8490,25 +8465,25 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="36" t="s">
+      <c r="D44" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="37"/>
-      <c r="F44" s="37"/>
-      <c r="G44" s="37"/>
-      <c r="H44" s="38"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40"/>
+      <c r="G44" s="40"/>
+      <c r="H44" s="41"/>
     </row>
     <row r="45" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
-      <c r="D45" s="36" t="s">
+      <c r="D45" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="E45" s="37"/>
-      <c r="F45" s="37"/>
-      <c r="G45" s="37"/>
-      <c r="H45" s="38"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="41"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
@@ -8532,25 +8507,25 @@
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="36" t="s">
+      <c r="D47" s="39" t="s">
         <v>145</v>
       </c>
-      <c r="E47" s="37"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="37"/>
-      <c r="H47" s="38"/>
+      <c r="E47" s="40"/>
+      <c r="F47" s="40"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="41"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="D48" s="36" t="s">
+      <c r="D48" s="39" t="s">
         <v>146</v>
       </c>
-      <c r="E48" s="37"/>
-      <c r="F48" s="37"/>
-      <c r="G48" s="37"/>
-      <c r="H48" s="38"/>
+      <c r="E48" s="40"/>
+      <c r="F48" s="40"/>
+      <c r="G48" s="40"/>
+      <c r="H48" s="41"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -8562,61 +8537,61 @@
       <c r="C49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D49" s="46" t="s">
+      <c r="D49" s="55" t="s">
         <v>278</v>
       </c>
-      <c r="E49" s="47"/>
-      <c r="F49" s="47"/>
-      <c r="G49" s="47"/>
-      <c r="H49" s="48"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="57"/>
     </row>
     <row r="50" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="D50" s="36" t="s">
+      <c r="D50" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="E50" s="37"/>
-      <c r="F50" s="37"/>
-      <c r="G50" s="37"/>
-      <c r="H50" s="38"/>
+      <c r="E50" s="40"/>
+      <c r="F50" s="40"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="41"/>
     </row>
     <row r="51" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="36" t="s">
+      <c r="D51" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="E51" s="37"/>
-      <c r="F51" s="37"/>
-      <c r="G51" s="37"/>
-      <c r="H51" s="38"/>
+      <c r="E51" s="40"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="41"/>
     </row>
     <row r="52" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="36" t="s">
+      <c r="D52" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="E52" s="37"/>
-      <c r="F52" s="37"/>
-      <c r="G52" s="37"/>
-      <c r="H52" s="38"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="40"/>
+      <c r="G52" s="40"/>
+      <c r="H52" s="41"/>
     </row>
     <row r="53" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
-      <c r="D53" s="36" t="s">
+      <c r="D53" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="E53" s="37"/>
-      <c r="F53" s="37"/>
-      <c r="G53" s="37"/>
-      <c r="H53" s="38"/>
+      <c r="E53" s="40"/>
+      <c r="F53" s="40"/>
+      <c r="G53" s="40"/>
+      <c r="H53" s="41"/>
     </row>
     <row r="54" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
@@ -8632,6 +8607,39 @@
     </row>
   </sheetData>
   <mergeCells count="49">
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D8:H8"/>
@@ -8648,39 +8656,6 @@
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="D22:H22"/>
     <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D49:H49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -8723,13 +8698,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -8783,13 +8758,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8981,13 +8956,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="42" t="s">
         <v>349</v>
       </c>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="45"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="44"/>
     </row>
     <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -9267,24 +9242,15 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
     <mergeCell ref="D34:H34"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D22:H22"/>
@@ -9299,15 +9265,24 @@
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9348,13 +9323,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -9408,13 +9383,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -9822,25 +9797,25 @@
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="36" t="s">
+      <c r="D39" s="39" t="s">
         <v>356</v>
       </c>
-      <c r="E39" s="37"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="37"/>
-      <c r="H39" s="38"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="40"/>
+      <c r="H39" s="41"/>
     </row>
     <row r="40" spans="1:8" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="36" t="s">
+      <c r="D40" s="39" t="s">
         <v>357</v>
       </c>
-      <c r="E40" s="37"/>
-      <c r="F40" s="37"/>
-      <c r="G40" s="37"/>
-      <c r="H40" s="38"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="40"/>
+      <c r="H40" s="41"/>
     </row>
     <row r="41" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -10017,25 +9992,22 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D36:H36"/>
     <mergeCell ref="D31:H31"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D52:H52"/>
@@ -10052,22 +10024,25 @@
     <mergeCell ref="D45:H45"/>
     <mergeCell ref="D46:H46"/>
     <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -10131,13 +10106,13 @@
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="36" t="s">
         <v>205</v>
       </c>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="42"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -10389,13 +10364,13 @@
       <c r="A24" s="12"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="42" t="s">
         <v>206</v>
       </c>
-      <c r="E24" s="44"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="45"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="43"/>
+      <c r="H24" s="44"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="12"/>
@@ -10795,12 +10770,40 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D8:H8"/>
     <mergeCell ref="D9:H9"/>
@@ -10813,40 +10816,12 @@
     <mergeCell ref="D16:H16"/>
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: leer excel del form manualmente + DisableAntiforgery para evitar error de antiforgery middleware
</commit_message>
<xml_diff>
--- a/apiService/Plantilla-modelo.xlsx
+++ b/apiService/Plantilla-modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollo-software\reporte-obras-main\apiService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D028D76E-691B-4511-ABA5-2A2A7ECF76E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE78089-98EC-4C67-964A-20EBB14FF31F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="947" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1449,7 +1449,7 @@
     <t>4.4 Verificar seguridades (FOTOS del cuadro antes y después).</t>
   </si>
   <si>
-    <t xml:space="preserve">4.3.1 PRUEBA </t>
+    <t xml:space="preserve">4.3 PRUEBA </t>
   </si>
 </sst>
 </file>
@@ -1712,6 +1712,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1721,12 +1724,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1736,6 +1733,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1744,15 +1744,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1780,6 +1771,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -2159,13 +2159,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -2195,13 +2195,13 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="48"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -2491,13 +2491,13 @@
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="49" t="s">
+      <c r="D27" s="48" t="s">
         <v>162</v>
       </c>
-      <c r="E27" s="50"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="51"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="50"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
@@ -2569,25 +2569,25 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="46" t="s">
+      <c r="D33" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="E33" s="47"/>
-      <c r="F33" s="47"/>
-      <c r="G33" s="47"/>
-      <c r="H33" s="48"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="43"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="44"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="14"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="42" t="s">
+      <c r="D34" s="45" t="s">
         <v>242</v>
       </c>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="44"/>
+      <c r="E34" s="46"/>
+      <c r="F34" s="46"/>
+      <c r="G34" s="46"/>
+      <c r="H34" s="47"/>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -2647,13 +2647,13 @@
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="42" t="s">
+      <c r="D39" s="45" t="s">
         <v>241</v>
       </c>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="E39" s="46"/>
+      <c r="F39" s="46"/>
+      <c r="G39" s="46"/>
+      <c r="H39" s="47"/>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -2806,6 +2806,32 @@
     <row r="282" ht="45" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D16:H16"/>
@@ -2822,32 +2848,6 @@
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D43:H43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3119,13 +3119,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="D4:H4"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D8:H8"/>
@@ -3138,6 +3131,13 @@
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="D4:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3180,13 +3180,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -3204,49 +3204,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="42" t="s">
         <v>362</v>
       </c>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="48"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="42" t="s">
         <v>363</v>
       </c>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="48"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="44"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -3438,85 +3438,85 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="42" t="s">
+      <c r="D22" s="45" t="s">
         <v>368</v>
       </c>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="44"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="47"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="42" t="s">
+      <c r="D23" s="45" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="44"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="47"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="42" t="s">
+      <c r="D24" s="45" t="s">
         <v>371</v>
       </c>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="47"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="42" t="s">
+      <c r="D25" s="45" t="s">
         <v>372</v>
       </c>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="44"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="47"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="42" t="s">
+      <c r="D26" s="45" t="s">
         <v>370</v>
       </c>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="44"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="47"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="12"/>
-      <c r="D27" s="42" t="s">
+      <c r="D27" s="45" t="s">
         <v>369</v>
       </c>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="47"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="12"/>
-      <c r="D28" s="42" t="s">
+      <c r="D28" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="44"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="47"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3552,13 +3552,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="42" t="s">
+      <c r="D31" s="45" t="s">
         <v>373</v>
       </c>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="44"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="47"/>
     </row>
     <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -3726,13 +3726,13 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="46" t="s">
+      <c r="D44" s="42" t="s">
         <v>102</v>
       </c>
-      <c r="E44" s="47"/>
-      <c r="F44" s="47"/>
-      <c r="G44" s="47"/>
-      <c r="H44" s="48"/>
+      <c r="E44" s="43"/>
+      <c r="F44" s="43"/>
+      <c r="G44" s="43"/>
+      <c r="H44" s="44"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
@@ -3750,25 +3750,25 @@
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
-      <c r="D46" s="46" t="s">
+      <c r="D46" s="42" t="s">
         <v>375</v>
       </c>
-      <c r="E46" s="47"/>
-      <c r="F46" s="47"/>
-      <c r="G46" s="47"/>
-      <c r="H46" s="48"/>
+      <c r="E46" s="43"/>
+      <c r="F46" s="43"/>
+      <c r="G46" s="43"/>
+      <c r="H46" s="44"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="46" t="s">
+      <c r="D47" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="E47" s="47"/>
-      <c r="F47" s="47"/>
-      <c r="G47" s="47"/>
-      <c r="H47" s="48"/>
+      <c r="E47" s="43"/>
+      <c r="F47" s="43"/>
+      <c r="G47" s="43"/>
+      <c r="H47" s="44"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3912,13 +3912,13 @@
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
-      <c r="D58" s="49" t="s">
+      <c r="D58" s="48" t="s">
         <v>114</v>
       </c>
-      <c r="E58" s="50"/>
-      <c r="F58" s="50"/>
-      <c r="G58" s="50"/>
-      <c r="H58" s="51"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="49"/>
+      <c r="G58" s="49"/>
+      <c r="H58" s="50"/>
     </row>
     <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
@@ -4342,24 +4342,61 @@
     </row>
   </sheetData>
   <mergeCells count="89">
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D87:H87"/>
+    <mergeCell ref="D88:H88"/>
+    <mergeCell ref="D89:H89"/>
+    <mergeCell ref="D74:H74"/>
+    <mergeCell ref="D63:H63"/>
+    <mergeCell ref="D64:H64"/>
+    <mergeCell ref="D65:H65"/>
+    <mergeCell ref="D66:H66"/>
+    <mergeCell ref="D67:H67"/>
+    <mergeCell ref="D68:H68"/>
+    <mergeCell ref="D69:H69"/>
+    <mergeCell ref="D70:H70"/>
+    <mergeCell ref="D71:H71"/>
+    <mergeCell ref="D72:H72"/>
+    <mergeCell ref="D90:H90"/>
+    <mergeCell ref="D91:H91"/>
+    <mergeCell ref="D86:H86"/>
+    <mergeCell ref="D75:H75"/>
+    <mergeCell ref="D76:H76"/>
+    <mergeCell ref="D77:H77"/>
+    <mergeCell ref="D78:H78"/>
+    <mergeCell ref="D79:H79"/>
+    <mergeCell ref="D80:H80"/>
+    <mergeCell ref="D81:H81"/>
+    <mergeCell ref="D82:H82"/>
+    <mergeCell ref="D83:H83"/>
+    <mergeCell ref="D84:H84"/>
+    <mergeCell ref="D85:H85"/>
+    <mergeCell ref="D73:H73"/>
+    <mergeCell ref="D62:H62"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
     <mergeCell ref="D37:H37"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D21:H21"/>
@@ -4376,61 +4413,24 @@
     <mergeCell ref="D25:H25"/>
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D73:H73"/>
-    <mergeCell ref="D62:H62"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D56:H56"/>
-    <mergeCell ref="D57:H57"/>
-    <mergeCell ref="D58:H58"/>
-    <mergeCell ref="D59:H59"/>
-    <mergeCell ref="D60:H60"/>
-    <mergeCell ref="D61:H61"/>
-    <mergeCell ref="D90:H90"/>
-    <mergeCell ref="D91:H91"/>
-    <mergeCell ref="D86:H86"/>
-    <mergeCell ref="D75:H75"/>
-    <mergeCell ref="D76:H76"/>
-    <mergeCell ref="D77:H77"/>
-    <mergeCell ref="D78:H78"/>
-    <mergeCell ref="D79:H79"/>
-    <mergeCell ref="D80:H80"/>
-    <mergeCell ref="D81:H81"/>
-    <mergeCell ref="D82:H82"/>
-    <mergeCell ref="D83:H83"/>
-    <mergeCell ref="D84:H84"/>
-    <mergeCell ref="D85:H85"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D87:H87"/>
-    <mergeCell ref="D88:H88"/>
-    <mergeCell ref="D89:H89"/>
-    <mergeCell ref="D74:H74"/>
-    <mergeCell ref="D63:H63"/>
-    <mergeCell ref="D64:H64"/>
-    <mergeCell ref="D65:H65"/>
-    <mergeCell ref="D66:H66"/>
-    <mergeCell ref="D67:H67"/>
-    <mergeCell ref="D68:H68"/>
-    <mergeCell ref="D69:H69"/>
-    <mergeCell ref="D70:H70"/>
-    <mergeCell ref="D71:H71"/>
-    <mergeCell ref="D72:H72"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4472,13 +4472,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -4532,13 +4532,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -4730,13 +4730,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="49" t="s">
+      <c r="D22" s="48" t="s">
         <v>384</v>
       </c>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="51"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -5004,12 +5004,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
@@ -5022,28 +5038,12 @@
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5311,6 +5311,11 @@
     <row r="20" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
     <mergeCell ref="D12:H12"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="D2:H2"/>
@@ -5323,11 +5328,6 @@
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5370,13 +5370,13 @@
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="45" t="s">
+      <c r="D8" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="45"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="51"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -5430,13 +5430,13 @@
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="46" t="s">
+      <c r="D13" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="47"/>
-      <c r="F13" s="47"/>
-      <c r="G13" s="47"/>
-      <c r="H13" s="48"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="44"/>
     </row>
     <row r="14" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
@@ -5772,13 +5772,13 @@
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="49" t="s">
+      <c r="D39" s="48" t="s">
         <v>306</v>
       </c>
-      <c r="E39" s="50"/>
-      <c r="F39" s="50"/>
-      <c r="G39" s="50"/>
-      <c r="H39" s="51"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
+      <c r="G39" s="49"/>
+      <c r="H39" s="50"/>
     </row>
     <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
@@ -5892,13 +5892,13 @@
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="D48" s="42" t="s">
+      <c r="D48" s="45" t="s">
         <v>253</v>
       </c>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="E48" s="46"/>
+      <c r="F48" s="46"/>
+      <c r="G48" s="46"/>
+      <c r="H48" s="47"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
@@ -5916,25 +5916,25 @@
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="D50" s="42" t="s">
+      <c r="D50" s="45" t="s">
         <v>254</v>
       </c>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43"/>
-      <c r="H50" s="44"/>
+      <c r="E50" s="46"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="46"/>
+      <c r="H50" s="47"/>
     </row>
     <row r="51" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="42" t="s">
+      <c r="D51" s="45" t="s">
         <v>308</v>
       </c>
-      <c r="E51" s="43"/>
-      <c r="F51" s="43"/>
-      <c r="G51" s="43"/>
-      <c r="H51" s="44"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="46"/>
+      <c r="H51" s="47"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
@@ -6088,12 +6088,36 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="D59:H59"/>
+    <mergeCell ref="D60:H60"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D57:H57"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
@@ -6110,36 +6134,12 @@
     <mergeCell ref="D29:H29"/>
     <mergeCell ref="D30:H30"/>
     <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D58:H58"/>
-    <mergeCell ref="D59:H59"/>
-    <mergeCell ref="D60:H60"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D57:H57"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6186,13 +6186,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6210,49 +6210,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="42" t="s">
         <v>310</v>
       </c>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="48"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="42" t="s">
         <v>311</v>
       </c>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="48"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="44"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -6432,13 +6432,13 @@
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="42" t="s">
+      <c r="D21" s="45" t="s">
         <v>316</v>
       </c>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="47"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -6616,6 +6616,27 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="D2:H2"/>
@@ -6628,27 +6649,6 @@
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D11:H11"/>
     <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
   </mergeCells>
   <pageMargins left="0.70866141732283461" right="0.70866141732283461" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6691,13 +6691,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6751,13 +6751,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
@@ -6949,13 +6949,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="49" t="s">
+      <c r="D22" s="48" t="s">
         <v>295</v>
       </c>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="51"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -7057,13 +7057,13 @@
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
-      <c r="D30" s="42" t="s">
+      <c r="D30" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="47"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
@@ -7081,25 +7081,25 @@
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="42" t="s">
+      <c r="D32" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="44"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="46"/>
+      <c r="H32" s="47"/>
     </row>
     <row r="33" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="42" t="s">
+      <c r="D33" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="43"/>
-      <c r="H33" s="44"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="46"/>
+      <c r="G33" s="46"/>
+      <c r="H33" s="47"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
@@ -7223,12 +7223,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
     <mergeCell ref="D20:H20"/>
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
@@ -7241,28 +7257,12 @@
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="D18:H18"/>
     <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7305,13 +7305,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -7365,13 +7365,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -7563,61 +7563,61 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="49" t="s">
+      <c r="D22" s="48" t="s">
         <v>272</v>
       </c>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="51"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="49" t="s">
+      <c r="D23" s="48" t="s">
         <v>323</v>
       </c>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="51"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="50"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="48" t="s">
         <v>324</v>
       </c>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="51"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="50"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="49" t="s">
+      <c r="D25" s="48" t="s">
         <v>325</v>
       </c>
-      <c r="E25" s="50"/>
-      <c r="F25" s="50"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="51"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="50"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-      <c r="D26" s="49" t="s">
+      <c r="D26" s="48" t="s">
         <v>326</v>
       </c>
-      <c r="E26" s="50"/>
-      <c r="F26" s="50"/>
-      <c r="G26" s="50"/>
-      <c r="H26" s="51"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
+      <c r="H26" s="50"/>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
@@ -7719,13 +7719,13 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="42" t="s">
+      <c r="D34" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="44"/>
+      <c r="E34" s="46"/>
+      <c r="F34" s="46"/>
+      <c r="G34" s="46"/>
+      <c r="H34" s="47"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -7743,25 +7743,25 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
-      <c r="D36" s="42" t="s">
+      <c r="D36" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="44"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="47"/>
     </row>
     <row r="37" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="42" t="s">
+      <c r="D37" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="44"/>
+      <c r="E37" s="46"/>
+      <c r="F37" s="46"/>
+      <c r="G37" s="46"/>
+      <c r="H37" s="47"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -7885,34 +7885,6 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
     <mergeCell ref="D35:H35"/>
     <mergeCell ref="D36:H36"/>
     <mergeCell ref="D21:H21"/>
@@ -7929,6 +7901,34 @@
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7971,13 +7971,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -8031,13 +8031,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8319,13 +8319,13 @@
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-      <c r="D29" s="49" t="s">
+      <c r="D29" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="50"/>
-      <c r="F29" s="50"/>
-      <c r="G29" s="50"/>
-      <c r="H29" s="51"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="50"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -8355,13 +8355,13 @@
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="58" t="s">
+      <c r="D32" s="55" t="s">
         <v>334</v>
       </c>
-      <c r="E32" s="59"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="59"/>
-      <c r="H32" s="60"/>
+      <c r="E32" s="56"/>
+      <c r="F32" s="56"/>
+      <c r="G32" s="56"/>
+      <c r="H32" s="57"/>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
@@ -8381,25 +8381,25 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="61" t="s">
+      <c r="D34" s="58" t="s">
         <v>335</v>
       </c>
-      <c r="E34" s="62"/>
-      <c r="F34" s="62"/>
-      <c r="G34" s="62"/>
-      <c r="H34" s="63"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="59"/>
+      <c r="G34" s="59"/>
+      <c r="H34" s="60"/>
     </row>
     <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
-      <c r="D35" s="64" t="s">
+      <c r="D35" s="61" t="s">
         <v>337</v>
       </c>
-      <c r="E35" s="65"/>
-      <c r="F35" s="65"/>
-      <c r="G35" s="65"/>
-      <c r="H35" s="66"/>
+      <c r="E35" s="62"/>
+      <c r="F35" s="62"/>
+      <c r="G35" s="62"/>
+      <c r="H35" s="63"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -8423,13 +8423,13 @@
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="42" t="s">
+      <c r="D37" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="44"/>
+      <c r="E37" s="46"/>
+      <c r="F37" s="46"/>
+      <c r="G37" s="46"/>
+      <c r="H37" s="47"/>
     </row>
     <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
@@ -8489,13 +8489,13 @@
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="42" t="s">
+      <c r="D42" s="45" t="s">
         <v>274</v>
       </c>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="43"/>
-      <c r="H42" s="44"/>
+      <c r="E42" s="46"/>
+      <c r="F42" s="46"/>
+      <c r="G42" s="46"/>
+      <c r="H42" s="47"/>
     </row>
     <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
@@ -8513,25 +8513,25 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="42" t="s">
+      <c r="D44" s="45" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="43"/>
-      <c r="F44" s="43"/>
-      <c r="G44" s="43"/>
-      <c r="H44" s="44"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
+      <c r="H44" s="47"/>
     </row>
     <row r="45" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
-      <c r="D45" s="42" t="s">
+      <c r="D45" s="45" t="s">
         <v>276</v>
       </c>
-      <c r="E45" s="43"/>
-      <c r="F45" s="43"/>
-      <c r="G45" s="43"/>
-      <c r="H45" s="44"/>
+      <c r="E45" s="46"/>
+      <c r="F45" s="46"/>
+      <c r="G45" s="46"/>
+      <c r="H45" s="47"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
@@ -8555,25 +8555,25 @@
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="42" t="s">
+      <c r="D47" s="45" t="s">
         <v>145</v>
       </c>
-      <c r="E47" s="43"/>
-      <c r="F47" s="43"/>
-      <c r="G47" s="43"/>
-      <c r="H47" s="44"/>
+      <c r="E47" s="46"/>
+      <c r="F47" s="46"/>
+      <c r="G47" s="46"/>
+      <c r="H47" s="47"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="D48" s="42" t="s">
+      <c r="D48" s="45" t="s">
         <v>146</v>
       </c>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="E48" s="46"/>
+      <c r="F48" s="46"/>
+      <c r="G48" s="46"/>
+      <c r="H48" s="47"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -8585,61 +8585,61 @@
       <c r="C49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D49" s="55" t="s">
+      <c r="D49" s="64" t="s">
         <v>278</v>
       </c>
-      <c r="E49" s="56"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="56"/>
-      <c r="H49" s="57"/>
+      <c r="E49" s="65"/>
+      <c r="F49" s="65"/>
+      <c r="G49" s="65"/>
+      <c r="H49" s="66"/>
     </row>
     <row r="50" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="D50" s="42" t="s">
+      <c r="D50" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43"/>
-      <c r="H50" s="44"/>
+      <c r="E50" s="46"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="46"/>
+      <c r="H50" s="47"/>
     </row>
     <row r="51" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="42" t="s">
+      <c r="D51" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="E51" s="43"/>
-      <c r="F51" s="43"/>
-      <c r="G51" s="43"/>
-      <c r="H51" s="44"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="46"/>
+      <c r="H51" s="47"/>
     </row>
     <row r="52" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="42" t="s">
+      <c r="D52" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="E52" s="43"/>
-      <c r="F52" s="43"/>
-      <c r="G52" s="43"/>
-      <c r="H52" s="44"/>
+      <c r="E52" s="46"/>
+      <c r="F52" s="46"/>
+      <c r="G52" s="46"/>
+      <c r="H52" s="47"/>
     </row>
     <row r="53" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
-      <c r="D53" s="42" t="s">
+      <c r="D53" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="E53" s="43"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="44"/>
+      <c r="E53" s="46"/>
+      <c r="F53" s="46"/>
+      <c r="G53" s="46"/>
+      <c r="H53" s="47"/>
     </row>
     <row r="54" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
@@ -8655,6 +8655,39 @@
     </row>
   </sheetData>
   <mergeCells count="49">
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="D8:H8"/>
@@ -8671,39 +8704,6 @@
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="D22:H22"/>
     <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="D49:H49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -8746,13 +8746,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -8806,13 +8806,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -9004,13 +9004,13 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="49" t="s">
+      <c r="D22" s="48" t="s">
         <v>346</v>
       </c>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="51"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -9290,24 +9290,15 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D16:H16"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
     <mergeCell ref="D34:H34"/>
     <mergeCell ref="D21:H21"/>
     <mergeCell ref="D22:H22"/>
@@ -9322,15 +9313,24 @@
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9371,13 +9371,13 @@
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -9431,13 +9431,13 @@
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -9845,25 +9845,25 @@
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="42" t="s">
+      <c r="D39" s="45" t="s">
         <v>353</v>
       </c>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="E39" s="46"/>
+      <c r="F39" s="46"/>
+      <c r="G39" s="46"/>
+      <c r="H39" s="47"/>
     </row>
     <row r="40" spans="1:8" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="42" t="s">
+      <c r="D40" s="45" t="s">
         <v>354</v>
       </c>
-      <c r="E40" s="43"/>
-      <c r="F40" s="43"/>
-      <c r="G40" s="43"/>
-      <c r="H40" s="44"/>
+      <c r="E40" s="46"/>
+      <c r="F40" s="46"/>
+      <c r="G40" s="46"/>
+      <c r="H40" s="47"/>
     </row>
     <row r="41" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -10040,25 +10040,22 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="D15:H15"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D36:H36"/>
     <mergeCell ref="D31:H31"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D52:H52"/>
@@ -10075,22 +10072,25 @@
     <mergeCell ref="D45:H45"/>
     <mergeCell ref="D46:H46"/>
     <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D14:H14"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D13:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -10154,13 +10154,13 @@
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="42" t="s">
         <v>205</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -10412,13 +10412,13 @@
       <c r="A24" s="12"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="48" t="s">
         <v>206</v>
       </c>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="51"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="50"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="12"/>
@@ -10818,12 +10818,40 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D22:H22"/>
+    <mergeCell ref="D23:H23"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="D26:H26"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
     <mergeCell ref="D19:H19"/>
     <mergeCell ref="D8:H8"/>
     <mergeCell ref="D9:H9"/>
@@ -10836,40 +10864,12 @@
     <mergeCell ref="D16:H16"/>
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D26:H26"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D38:H38"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: corregir faltas ortograficas en config-centros (obserbar->observar, solidos->sólidos)
</commit_message>
<xml_diff>
--- a/apiService/Plantilla-modelo.xlsx
+++ b/apiService/Plantilla-modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollo-software\reporte-obras-main\apiService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE78089-98EC-4C67-964A-20EBB14FF31F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B01C328-F109-4930-A526-F1DA8DAE7439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="947" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1449,7 +1449,7 @@
     <t>4.4 Verificar seguridades (FOTOS del cuadro antes y después).</t>
   </si>
   <si>
-    <t xml:space="preserve">4.3 PRUEBA </t>
+    <t>4.5 PRUEBA NUMERO 20000</t>
   </si>
 </sst>
 </file>
@@ -1607,7 +1607,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1664,8 +1664,8 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1782,6 +1782,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5051,7 +5063,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6D5BD9-6748-4A03-A6F1-166697746BD8}">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
@@ -5289,7 +5301,7 @@
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="26" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E18" s="21"/>
       <c r="F18" s="21"/>
@@ -5300,15 +5312,35 @@
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="4" t="s">
-        <v>393</v>
+      <c r="D19" s="26" t="s">
+        <v>394</v>
       </c>
       <c r="E19" s="21"/>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
       <c r="H19" s="22"/>
     </row>
-    <row r="20" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="68"/>
+      <c r="B20" s="68"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="70"/>
+      <c r="F20" s="70"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="70"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="68"/>
+      <c r="B21" s="68"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="69"/>
+      <c r="E21" s="70"/>
+      <c r="F21" s="70"/>
+      <c r="G21" s="70"/>
+      <c r="H21" s="70"/>
+    </row>
+    <row r="22" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="D15:H15"/>

</xml_diff>

<commit_message>
Primera prueba de mejora de sincro
</commit_message>
<xml_diff>
--- a/apiService/Plantilla-modelo.xlsx
+++ b/apiService/Plantilla-modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollo-software\reporte-obras-main\apiService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A05944F5-7EE6-4F2D-A4A6-1AB9F9A72972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD7BD6C-F904-4858-87E9-F28C4C5D96A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="947" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="397">
   <si>
     <t>REVISADO</t>
   </si>
@@ -1411,6 +1411,9 @@
   </si>
   <si>
     <t>5.3 Vaciar neutralizador 1 completamente y observar el estado de mangueras, acoples, solidos en el fondo… (FOTOS)</t>
+  </si>
+  <si>
+    <t>8.6 Prueba de sincro numero 2</t>
   </si>
 </sst>
 </file>
@@ -1643,14 +1646,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1661,6 +1664,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1671,6 +1689,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1678,30 +1705,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2114,25 +2117,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -2162,13 +2165,13 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="48" t="s">
+      <c r="D5" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="50"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -2180,13 +2183,13 @@
       <c r="C6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="38" t="s">
         <v>149</v>
       </c>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="34"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="40"/>
     </row>
     <row r="7" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
@@ -2216,13 +2219,13 @@
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
-      <c r="H9" s="40"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="47"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
@@ -2274,13 +2277,13 @@
       <c r="C13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="38" t="s">
         <v>218</v>
       </c>
-      <c r="E13" s="33"/>
-      <c r="F13" s="33"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="34"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="40"/>
     </row>
     <row r="14" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -2310,13 +2313,13 @@
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="40"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="47"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
@@ -2368,13 +2371,13 @@
       <c r="C20" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D20" s="38" t="s">
         <v>219</v>
       </c>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="34"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="40"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
@@ -2446,25 +2449,25 @@
       <c r="C26" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="32" t="s">
+      <c r="D26" s="38" t="s">
         <v>220</v>
       </c>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="34"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="40"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="51" t="s">
+      <c r="D27" s="48" t="s">
         <v>152</v>
       </c>
-      <c r="E27" s="52"/>
-      <c r="F27" s="52"/>
-      <c r="G27" s="52"/>
-      <c r="H27" s="53"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="50"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
@@ -2500,13 +2503,13 @@
       <c r="C30" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D30" s="32" t="s">
+      <c r="D30" s="38" t="s">
         <v>181</v>
       </c>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="34"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="40"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
@@ -2536,25 +2539,25 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="48" t="s">
+      <c r="D33" s="42" t="s">
         <v>146</v>
       </c>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="50"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="43"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="44"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="14"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="44" t="s">
+      <c r="D34" s="32" t="s">
         <v>226</v>
       </c>
-      <c r="E34" s="45"/>
-      <c r="F34" s="45"/>
-      <c r="G34" s="45"/>
-      <c r="H34" s="46"/>
+      <c r="E34" s="33"/>
+      <c r="F34" s="33"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="34"/>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -2566,13 +2569,13 @@
       <c r="C35" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D35" s="32" t="s">
+      <c r="D35" s="38" t="s">
         <v>221</v>
       </c>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="34"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="39"/>
+      <c r="H35" s="40"/>
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
@@ -2614,13 +2617,13 @@
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="44" t="s">
+      <c r="D39" s="32" t="s">
         <v>225</v>
       </c>
-      <c r="E39" s="45"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="45"/>
-      <c r="H39" s="46"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="33"/>
+      <c r="H39" s="34"/>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -2632,13 +2635,13 @@
       <c r="C40" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="32" t="s">
+      <c r="D40" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33"/>
-      <c r="G40" s="33"/>
-      <c r="H40" s="34"/>
+      <c r="E40" s="39"/>
+      <c r="F40" s="39"/>
+      <c r="G40" s="39"/>
+      <c r="H40" s="40"/>
     </row>
     <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -2674,13 +2677,13 @@
       <c r="C43" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D43" s="32" t="s">
+      <c r="D43" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E43" s="33"/>
-      <c r="F43" s="33"/>
-      <c r="G43" s="33"/>
-      <c r="H43" s="34"/>
+      <c r="E43" s="39"/>
+      <c r="F43" s="39"/>
+      <c r="G43" s="39"/>
+      <c r="H43" s="40"/>
     </row>
     <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
@@ -2742,11 +2745,23 @@
       <c r="G48" s="30"/>
       <c r="H48" s="31"/>
     </row>
-    <row r="50" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="29" t="s">
+        <v>396</v>
+      </c>
+      <c r="E49" s="30"/>
+      <c r="F49" s="30"/>
+      <c r="G49" s="30"/>
+      <c r="H49" s="31"/>
+    </row>
+    <row r="50" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="105" ht="78.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="106" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="107" ht="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -2772,7 +2787,7 @@
     <row r="260" ht="25.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="282" ht="45" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="43">
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="D33:H33"/>
     <mergeCell ref="D16:H16"/>
@@ -2806,6 +2821,7 @@
     <mergeCell ref="D37:H37"/>
     <mergeCell ref="D38:H38"/>
     <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D49:H49"/>
     <mergeCell ref="D41:H41"/>
     <mergeCell ref="D42:H42"/>
     <mergeCell ref="D39:H39"/>
@@ -2842,13 +2858,13 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
@@ -2878,37 +2894,37 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="45" t="s">
         <v>216</v>
       </c>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="40"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="47"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>335</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>336</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="53"/>
     </row>
     <row r="7" spans="1:8" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
@@ -2932,13 +2948,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>261</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -2974,13 +2990,13 @@
       <c r="C11" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D11" s="32" t="s">
+      <c r="D11" s="38" t="s">
         <v>262</v>
       </c>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="34"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="40"/>
     </row>
     <row r="12" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
@@ -3016,13 +3032,13 @@
       <c r="C14" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="38" t="s">
         <v>263</v>
       </c>
-      <c r="E14" s="33"/>
-      <c r="F14" s="33"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="34"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="40"/>
     </row>
     <row r="15" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
@@ -3135,25 +3151,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -3171,49 +3187,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="48" t="s">
+      <c r="D4" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="50"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="48" t="s">
+      <c r="D5" s="42" t="s">
         <v>341</v>
       </c>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="50"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="48" t="s">
+      <c r="D6" s="42" t="s">
         <v>342</v>
       </c>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="50"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="44"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -3225,13 +3241,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -3261,37 +3277,37 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>343</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>344</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -3315,13 +3331,13 @@
       <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="40"/>
     </row>
     <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -3393,97 +3409,97 @@
       <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40"/>
     </row>
     <row r="22" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="44" t="s">
+      <c r="D22" s="32" t="s">
         <v>347</v>
       </c>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="46"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="34"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="44" t="s">
+      <c r="D23" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="46"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="34"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="44" t="s">
+      <c r="D24" s="32" t="s">
         <v>350</v>
       </c>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="46"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="34"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="44" t="s">
+      <c r="D25" s="32" t="s">
         <v>351</v>
       </c>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="46"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="34"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="44" t="s">
+      <c r="D26" s="32" t="s">
         <v>349</v>
       </c>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="46"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="34"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="12"/>
-      <c r="D27" s="44" t="s">
+      <c r="D27" s="32" t="s">
         <v>348</v>
       </c>
-      <c r="E27" s="45"/>
-      <c r="F27" s="45"/>
-      <c r="G27" s="45"/>
-      <c r="H27" s="46"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="34"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="12"/>
-      <c r="D28" s="44" t="s">
+      <c r="D28" s="32" t="s">
         <v>217</v>
       </c>
-      <c r="E28" s="45"/>
-      <c r="F28" s="45"/>
-      <c r="G28" s="45"/>
-      <c r="H28" s="46"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="34"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3495,13 +3511,13 @@
       <c r="C29" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="34"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="40"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -3519,13 +3535,13 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="44" t="s">
+      <c r="D31" s="32" t="s">
         <v>352</v>
       </c>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
-      <c r="G31" s="45"/>
-      <c r="H31" s="46"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="34"/>
     </row>
     <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -3561,13 +3577,13 @@
       <c r="C34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D34" s="32" t="s">
+      <c r="D34" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="34"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="40"/>
     </row>
     <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -3627,13 +3643,13 @@
       <c r="C39" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D39" s="32" t="s">
+      <c r="D39" s="38" t="s">
         <v>93</v>
       </c>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-      <c r="G39" s="33"/>
-      <c r="H39" s="34"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="39"/>
+      <c r="G39" s="39"/>
+      <c r="H39" s="40"/>
     </row>
     <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
@@ -3669,13 +3685,13 @@
       <c r="C42" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D42" s="32" t="s">
+      <c r="D42" s="38" t="s">
         <v>95</v>
       </c>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="34"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="39"/>
+      <c r="G42" s="39"/>
+      <c r="H42" s="40"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
@@ -3693,13 +3709,13 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="48" t="s">
+      <c r="D44" s="42" t="s">
         <v>97</v>
       </c>
-      <c r="E44" s="49"/>
-      <c r="F44" s="49"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="50"/>
+      <c r="E44" s="43"/>
+      <c r="F44" s="43"/>
+      <c r="G44" s="43"/>
+      <c r="H44" s="44"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
@@ -3717,25 +3733,25 @@
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
-      <c r="D46" s="48" t="s">
+      <c r="D46" s="42" t="s">
         <v>354</v>
       </c>
-      <c r="E46" s="49"/>
-      <c r="F46" s="49"/>
-      <c r="G46" s="49"/>
-      <c r="H46" s="50"/>
+      <c r="E46" s="43"/>
+      <c r="F46" s="43"/>
+      <c r="G46" s="43"/>
+      <c r="H46" s="44"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="48" t="s">
+      <c r="D47" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="E47" s="49"/>
-      <c r="F47" s="49"/>
-      <c r="G47" s="49"/>
-      <c r="H47" s="50"/>
+      <c r="E47" s="43"/>
+      <c r="F47" s="43"/>
+      <c r="G47" s="43"/>
+      <c r="H47" s="44"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3747,13 +3763,13 @@
       <c r="C48" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D48" s="32" t="s">
+      <c r="D48" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="E48" s="33"/>
-      <c r="F48" s="33"/>
-      <c r="G48" s="33"/>
-      <c r="H48" s="34"/>
+      <c r="E48" s="39"/>
+      <c r="F48" s="39"/>
+      <c r="G48" s="39"/>
+      <c r="H48" s="40"/>
     </row>
     <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
@@ -3801,13 +3817,13 @@
       <c r="C52" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D52" s="32" t="s">
+      <c r="D52" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="E52" s="33"/>
-      <c r="F52" s="33"/>
-      <c r="G52" s="33"/>
-      <c r="H52" s="34"/>
+      <c r="E52" s="39"/>
+      <c r="F52" s="39"/>
+      <c r="G52" s="39"/>
+      <c r="H52" s="40"/>
     </row>
     <row r="53" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
@@ -3867,25 +3883,25 @@
       <c r="C57" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D57" s="32" t="s">
+      <c r="D57" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="E57" s="33"/>
-      <c r="F57" s="33"/>
-      <c r="G57" s="33"/>
-      <c r="H57" s="34"/>
+      <c r="E57" s="39"/>
+      <c r="F57" s="39"/>
+      <c r="G57" s="39"/>
+      <c r="H57" s="40"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
-      <c r="D58" s="51" t="s">
+      <c r="D58" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="52"/>
-      <c r="H58" s="53"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="49"/>
+      <c r="G58" s="49"/>
+      <c r="H58" s="50"/>
     </row>
     <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
@@ -3933,13 +3949,13 @@
       <c r="C62" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D62" s="32" t="s">
+      <c r="D62" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="E62" s="33"/>
-      <c r="F62" s="33"/>
-      <c r="G62" s="33"/>
-      <c r="H62" s="34"/>
+      <c r="E62" s="39"/>
+      <c r="F62" s="39"/>
+      <c r="G62" s="39"/>
+      <c r="H62" s="40"/>
     </row>
     <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
@@ -4071,13 +4087,13 @@
       <c r="C73" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D73" s="32" t="s">
+      <c r="D73" s="38" t="s">
         <v>123</v>
       </c>
-      <c r="E73" s="33"/>
-      <c r="F73" s="33"/>
-      <c r="G73" s="33"/>
-      <c r="H73" s="34"/>
+      <c r="E73" s="39"/>
+      <c r="F73" s="39"/>
+      <c r="G73" s="39"/>
+      <c r="H73" s="40"/>
     </row>
     <row r="74" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
@@ -4149,13 +4165,13 @@
       <c r="C79" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D79" s="32" t="s">
+      <c r="D79" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="E79" s="33"/>
-      <c r="F79" s="33"/>
-      <c r="G79" s="33"/>
-      <c r="H79" s="34"/>
+      <c r="E79" s="39"/>
+      <c r="F79" s="39"/>
+      <c r="G79" s="39"/>
+      <c r="H79" s="40"/>
     </row>
     <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
@@ -4185,37 +4201,37 @@
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
-      <c r="D82" s="38" t="s">
+      <c r="D82" s="45" t="s">
         <v>128</v>
       </c>
-      <c r="E82" s="39"/>
-      <c r="F82" s="39"/>
-      <c r="G82" s="39"/>
-      <c r="H82" s="40"/>
+      <c r="E82" s="46"/>
+      <c r="F82" s="46"/>
+      <c r="G82" s="46"/>
+      <c r="H82" s="47"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
-      <c r="D83" s="41" t="s">
+      <c r="D83" s="51" t="s">
         <v>356</v>
       </c>
-      <c r="E83" s="42"/>
-      <c r="F83" s="42"/>
-      <c r="G83" s="42"/>
-      <c r="H83" s="43"/>
+      <c r="E83" s="52"/>
+      <c r="F83" s="52"/>
+      <c r="G83" s="52"/>
+      <c r="H83" s="53"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
-      <c r="D84" s="41" t="s">
+      <c r="D84" s="51" t="s">
         <v>357</v>
       </c>
-      <c r="E84" s="42"/>
-      <c r="F84" s="42"/>
-      <c r="G84" s="42"/>
-      <c r="H84" s="43"/>
+      <c r="E84" s="52"/>
+      <c r="F84" s="52"/>
+      <c r="G84" s="52"/>
+      <c r="H84" s="53"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
@@ -4239,13 +4255,13 @@
       <c r="C86" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D86" s="32" t="s">
+      <c r="D86" s="38" t="s">
         <v>129</v>
       </c>
-      <c r="E86" s="33"/>
-      <c r="F86" s="33"/>
-      <c r="G86" s="33"/>
-      <c r="H86" s="34"/>
+      <c r="E86" s="39"/>
+      <c r="F86" s="39"/>
+      <c r="G86" s="39"/>
+      <c r="H86" s="40"/>
     </row>
     <row r="87" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A87" s="2"/>
@@ -4427,25 +4443,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -4475,37 +4491,37 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>307</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>358</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="53"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -4517,13 +4533,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -4553,37 +4569,37 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>359</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>360</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -4607,13 +4623,13 @@
       <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="38" t="s">
         <v>135</v>
       </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="40"/>
     </row>
     <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -4685,25 +4701,25 @@
       <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40"/>
     </row>
     <row r="22" spans="1:8" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="51" t="s">
+      <c r="D22" s="48" t="s">
         <v>363</v>
       </c>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="53"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -4739,13 +4755,13 @@
       <c r="C25" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D25" s="32" t="s">
+      <c r="D25" s="38" t="s">
         <v>136</v>
       </c>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="34"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="40"/>
     </row>
     <row r="26" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
@@ -4793,13 +4809,13 @@
       <c r="C29" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="38" t="s">
         <v>137</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="34"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="40"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -4859,13 +4875,13 @@
       <c r="C34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D34" s="32" t="s">
+      <c r="D34" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="34"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="40"/>
     </row>
     <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -4901,13 +4917,13 @@
       <c r="C37" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D37" s="32" t="s">
+      <c r="D37" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="33"/>
-      <c r="H37" s="34"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="40"/>
     </row>
     <row r="38" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
@@ -5031,13 +5047,13 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
@@ -5067,37 +5083,37 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="45" t="s">
         <v>216</v>
       </c>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="40"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="47"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>364</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>365</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="53"/>
     </row>
     <row r="7" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
@@ -5121,13 +5137,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>261</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -5163,13 +5179,13 @@
       <c r="C11" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D11" s="32" t="s">
+      <c r="D11" s="38" t="s">
         <v>262</v>
       </c>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="34"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="40"/>
     </row>
     <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
@@ -5207,13 +5223,13 @@
       <c r="C14" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="38" t="s">
         <v>263</v>
       </c>
-      <c r="E14" s="33"/>
-      <c r="F14" s="33"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="34"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="40"/>
     </row>
     <row r="15" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
@@ -5345,25 +5361,25 @@
       <c r="C7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="D7" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="34"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="40"/>
     </row>
     <row r="8" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="47" t="s">
+      <c r="D8" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="41"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -5393,37 +5409,37 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="51" t="s">
         <v>277</v>
       </c>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="43"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="53"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>278</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="48" t="s">
+      <c r="D13" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="49"/>
-      <c r="H13" s="50"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="44"/>
     </row>
     <row r="14" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
@@ -5471,37 +5487,37 @@
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="40"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="47"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="51" t="s">
         <v>279</v>
       </c>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="43"/>
+      <c r="E18" s="52"/>
+      <c r="F18" s="52"/>
+      <c r="G18" s="52"/>
+      <c r="H18" s="53"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="51" t="s">
         <v>280</v>
       </c>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="43"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="53"/>
     </row>
     <row r="20" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
@@ -5525,13 +5541,13 @@
       <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="38" t="s">
         <v>227</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40"/>
     </row>
     <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
@@ -5561,37 +5577,37 @@
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
-      <c r="D24" s="38" t="s">
+      <c r="D24" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="40"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="47"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="51" t="s">
         <v>282</v>
       </c>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="43"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="52"/>
+      <c r="H25" s="53"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-      <c r="D26" s="41" t="s">
+      <c r="D26" s="51" t="s">
         <v>283</v>
       </c>
-      <c r="E26" s="42"/>
-      <c r="F26" s="42"/>
-      <c r="G26" s="42"/>
-      <c r="H26" s="43"/>
+      <c r="E26" s="52"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="53"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
@@ -5603,13 +5619,13 @@
       <c r="C27" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="32" t="s">
+      <c r="D27" s="38" t="s">
         <v>228</v>
       </c>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="34"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="40"/>
     </row>
     <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
@@ -5639,25 +5655,25 @@
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
-      <c r="D30" s="38" t="s">
+      <c r="D30" s="45" t="s">
         <v>176</v>
       </c>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="39"/>
-      <c r="H30" s="40"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="47"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="51" t="s">
         <v>284</v>
       </c>
-      <c r="E31" s="42"/>
-      <c r="F31" s="42"/>
-      <c r="G31" s="42"/>
-      <c r="H31" s="43"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="52"/>
+      <c r="H31" s="53"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
@@ -5669,13 +5685,13 @@
       <c r="C32" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D32" s="32" t="s">
+      <c r="D32" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="E32" s="33"/>
-      <c r="F32" s="33"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="34"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="39"/>
+      <c r="G32" s="39"/>
+      <c r="H32" s="40"/>
     </row>
     <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
@@ -5747,25 +5763,25 @@
       <c r="C38" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D38" s="32" t="s">
+      <c r="D38" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="33"/>
-      <c r="H38" s="34"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="40"/>
     </row>
     <row r="39" spans="1:8" ht="78.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="51" t="s">
+      <c r="D39" s="48" t="s">
         <v>287</v>
       </c>
-      <c r="E39" s="52"/>
-      <c r="F39" s="52"/>
-      <c r="G39" s="52"/>
-      <c r="H39" s="53"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
+      <c r="G39" s="49"/>
+      <c r="H39" s="50"/>
     </row>
     <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
@@ -5801,13 +5817,13 @@
       <c r="C42" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D42" s="32" t="s">
+      <c r="D42" s="38" t="s">
         <v>234</v>
       </c>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="34"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="39"/>
+      <c r="G42" s="39"/>
+      <c r="H42" s="40"/>
     </row>
     <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
@@ -5867,61 +5883,61 @@
       <c r="C47" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D47" s="32" t="s">
+      <c r="D47" s="38" t="s">
         <v>235</v>
       </c>
-      <c r="E47" s="33"/>
-      <c r="F47" s="33"/>
-      <c r="G47" s="33"/>
-      <c r="H47" s="34"/>
+      <c r="E47" s="39"/>
+      <c r="F47" s="39"/>
+      <c r="G47" s="39"/>
+      <c r="H47" s="40"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="D48" s="44" t="s">
+      <c r="D48" s="32" t="s">
         <v>236</v>
       </c>
-      <c r="E48" s="45"/>
-      <c r="F48" s="45"/>
-      <c r="G48" s="45"/>
-      <c r="H48" s="46"/>
+      <c r="E48" s="33"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="33"/>
+      <c r="H48" s="34"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
-      <c r="D49" s="41" t="s">
+      <c r="D49" s="51" t="s">
         <v>288</v>
       </c>
-      <c r="E49" s="42"/>
-      <c r="F49" s="42"/>
-      <c r="G49" s="42"/>
-      <c r="H49" s="43"/>
+      <c r="E49" s="52"/>
+      <c r="F49" s="52"/>
+      <c r="G49" s="52"/>
+      <c r="H49" s="53"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="D50" s="44" t="s">
+      <c r="D50" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="E50" s="45"/>
-      <c r="F50" s="45"/>
-      <c r="G50" s="45"/>
-      <c r="H50" s="46"/>
+      <c r="E50" s="33"/>
+      <c r="F50" s="33"/>
+      <c r="G50" s="33"/>
+      <c r="H50" s="34"/>
     </row>
     <row r="51" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="44" t="s">
+      <c r="D51" s="32" t="s">
         <v>374</v>
       </c>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
-      <c r="G51" s="45"/>
-      <c r="H51" s="46"/>
+      <c r="E51" s="33"/>
+      <c r="F51" s="33"/>
+      <c r="G51" s="33"/>
+      <c r="H51" s="34"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
@@ -5933,13 +5949,13 @@
       <c r="C52" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D52" s="32" t="s">
+      <c r="D52" s="38" t="s">
         <v>238</v>
       </c>
-      <c r="E52" s="33"/>
-      <c r="F52" s="33"/>
-      <c r="G52" s="33"/>
-      <c r="H52" s="34"/>
+      <c r="E52" s="39"/>
+      <c r="F52" s="39"/>
+      <c r="G52" s="39"/>
+      <c r="H52" s="40"/>
     </row>
     <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
@@ -5975,13 +5991,13 @@
       <c r="C55" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D55" s="32" t="s">
+      <c r="D55" s="38" t="s">
         <v>240</v>
       </c>
-      <c r="E55" s="33"/>
-      <c r="F55" s="33"/>
-      <c r="G55" s="33"/>
-      <c r="H55" s="34"/>
+      <c r="E55" s="39"/>
+      <c r="F55" s="39"/>
+      <c r="G55" s="39"/>
+      <c r="H55" s="40"/>
     </row>
     <row r="56" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
@@ -6161,25 +6177,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6197,49 +6213,49 @@
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="48" t="s">
+      <c r="D4" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="50"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="48" t="s">
+      <c r="D5" s="42" t="s">
         <v>290</v>
       </c>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="50"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="48" t="s">
+      <c r="D6" s="42" t="s">
         <v>291</v>
       </c>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="50"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="44"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -6251,13 +6267,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -6287,37 +6303,37 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
     </row>
     <row r="12" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>292</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>293</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -6341,13 +6357,13 @@
       <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="40"/>
     </row>
     <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -6407,25 +6423,25 @@
       <c r="C20" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D20" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="34"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="40"/>
     </row>
     <row r="21" spans="1:8" ht="65.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="44" t="s">
+      <c r="D21" s="32" t="s">
         <v>295</v>
       </c>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="46"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="34"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -6437,13 +6453,13 @@
       <c r="C22" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="32" t="s">
+      <c r="D22" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="34"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="40"/>
     </row>
     <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -6491,13 +6507,13 @@
       <c r="C26" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="32" t="s">
+      <c r="D26" s="38" t="s">
         <v>247</v>
       </c>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="34"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="40"/>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
@@ -6533,13 +6549,13 @@
       <c r="C29" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="38" t="s">
         <v>250</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="34"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="40"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -6666,25 +6682,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -6714,37 +6730,37 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>269</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>270</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="53"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
@@ -6792,37 +6808,37 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>271</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>272</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -6846,13 +6862,13 @@
       <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="40"/>
     </row>
     <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -6924,25 +6940,25 @@
       <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="38" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40"/>
     </row>
     <row r="22" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="51" t="s">
+      <c r="D22" s="48" t="s">
         <v>276</v>
       </c>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="53"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -6978,13 +6994,13 @@
       <c r="C25" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D25" s="32" t="s">
+      <c r="D25" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="34"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="40"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
@@ -7032,61 +7048,61 @@
       <c r="C29" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="34"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="40"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
-      <c r="D30" s="44" t="s">
+      <c r="D30" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
-      <c r="G30" s="45"/>
-      <c r="H30" s="46"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="34"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="51" t="s">
         <v>275</v>
       </c>
-      <c r="E31" s="42"/>
-      <c r="F31" s="42"/>
-      <c r="G31" s="42"/>
-      <c r="H31" s="43"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="52"/>
+      <c r="H31" s="53"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="44" t="s">
+      <c r="D32" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="45"/>
-      <c r="F32" s="45"/>
-      <c r="G32" s="45"/>
-      <c r="H32" s="46"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="34"/>
     </row>
     <row r="33" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="44" t="s">
+      <c r="D33" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="E33" s="45"/>
-      <c r="F33" s="45"/>
-      <c r="G33" s="45"/>
-      <c r="H33" s="46"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+      <c r="G33" s="33"/>
+      <c r="H33" s="34"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
@@ -7098,13 +7114,13 @@
       <c r="C34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D34" s="32" t="s">
+      <c r="D34" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="34"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="40"/>
     </row>
     <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
@@ -7140,13 +7156,13 @@
       <c r="C37" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D37" s="32" t="s">
+      <c r="D37" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="33"/>
-      <c r="H37" s="34"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="40"/>
     </row>
     <row r="38" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
@@ -7280,25 +7296,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -7328,37 +7344,37 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>296</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>297</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="53"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -7370,13 +7386,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -7406,37 +7422,37 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>298</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>299</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -7460,13 +7476,13 @@
       <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="40"/>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -7538,73 +7554,73 @@
       <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="51" t="s">
+      <c r="D22" s="48" t="s">
         <v>255</v>
       </c>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="53"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="51" t="s">
+      <c r="D23" s="48" t="s">
         <v>302</v>
       </c>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="52"/>
-      <c r="H23" s="53"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="50"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
-      <c r="D24" s="51" t="s">
+      <c r="D24" s="48" t="s">
         <v>303</v>
       </c>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="53"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="50"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="51" t="s">
+      <c r="D25" s="48" t="s">
         <v>304</v>
       </c>
-      <c r="E25" s="52"/>
-      <c r="F25" s="52"/>
-      <c r="G25" s="52"/>
-      <c r="H25" s="53"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="50"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-      <c r="D26" s="51" t="s">
+      <c r="D26" s="48" t="s">
         <v>305</v>
       </c>
-      <c r="E26" s="52"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="52"/>
-      <c r="H26" s="53"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
+      <c r="H26" s="50"/>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
@@ -7640,13 +7656,13 @@
       <c r="C29" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="34"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="40"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -7694,61 +7710,61 @@
       <c r="C33" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D33" s="32" t="s">
+      <c r="D33" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="E33" s="33"/>
-      <c r="F33" s="33"/>
-      <c r="G33" s="33"/>
-      <c r="H33" s="34"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="40"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="44" t="s">
+      <c r="D34" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="E34" s="45"/>
-      <c r="F34" s="45"/>
-      <c r="G34" s="45"/>
-      <c r="H34" s="46"/>
+      <c r="E34" s="33"/>
+      <c r="F34" s="33"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="34"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
-      <c r="D35" s="41" t="s">
+      <c r="D35" s="51" t="s">
         <v>306</v>
       </c>
-      <c r="E35" s="42"/>
-      <c r="F35" s="42"/>
-      <c r="G35" s="42"/>
-      <c r="H35" s="43"/>
+      <c r="E35" s="52"/>
+      <c r="F35" s="52"/>
+      <c r="G35" s="52"/>
+      <c r="H35" s="53"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
-      <c r="D36" s="44" t="s">
+      <c r="D36" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="E36" s="45"/>
-      <c r="F36" s="45"/>
-      <c r="G36" s="45"/>
-      <c r="H36" s="46"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="34"/>
     </row>
     <row r="37" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="44" t="s">
+      <c r="D37" s="32" t="s">
         <v>379</v>
       </c>
-      <c r="E37" s="45"/>
-      <c r="F37" s="45"/>
-      <c r="G37" s="45"/>
-      <c r="H37" s="46"/>
+      <c r="E37" s="33"/>
+      <c r="F37" s="33"/>
+      <c r="G37" s="33"/>
+      <c r="H37" s="34"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -7760,13 +7776,13 @@
       <c r="C38" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D38" s="32" t="s">
+      <c r="D38" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="33"/>
-      <c r="H38" s="34"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="40"/>
     </row>
     <row r="39" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
@@ -7802,13 +7818,13 @@
       <c r="C41" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D41" s="32" t="s">
+      <c r="D41" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E41" s="33"/>
-      <c r="F41" s="33"/>
-      <c r="G41" s="33"/>
-      <c r="H41" s="34"/>
+      <c r="E41" s="39"/>
+      <c r="F41" s="39"/>
+      <c r="G41" s="39"/>
+      <c r="H41" s="40"/>
     </row>
     <row r="42" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
@@ -7946,25 +7962,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -7994,37 +8010,37 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>307</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>308</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="53"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8036,13 +8052,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -8072,37 +8088,37 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>309</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>310</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -8126,13 +8142,13 @@
       <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="38" t="s">
         <v>218</v>
       </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="40"/>
     </row>
     <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -8162,37 +8178,37 @@
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
-      <c r="D18" s="38" t="s">
+      <c r="D18" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="40"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="47"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="51" t="s">
         <v>309</v>
       </c>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="43"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="53"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="51" t="s">
         <v>310</v>
       </c>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="43"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="53"/>
     </row>
     <row r="21" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
@@ -8216,13 +8232,13 @@
       <c r="C22" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="32" t="s">
+      <c r="D22" s="38" t="s">
         <v>256</v>
       </c>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="34"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="40"/>
     </row>
     <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -8294,25 +8310,25 @@
       <c r="C28" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D28" s="32" t="s">
+      <c r="D28" s="38" t="s">
         <v>220</v>
       </c>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="34"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="40"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-      <c r="D29" s="51" t="s">
+      <c r="D29" s="48" t="s">
         <v>63</v>
       </c>
-      <c r="E29" s="52"/>
-      <c r="F29" s="52"/>
-      <c r="G29" s="52"/>
-      <c r="H29" s="53"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="50"/>
     </row>
     <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -8398,25 +8414,25 @@
       <c r="C36" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D36" s="32" t="s">
+      <c r="D36" s="38" t="s">
         <v>181</v>
       </c>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="34"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
+      <c r="H36" s="40"/>
     </row>
     <row r="37" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="44" t="s">
+      <c r="D37" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="E37" s="45"/>
-      <c r="F37" s="45"/>
-      <c r="G37" s="45"/>
-      <c r="H37" s="46"/>
+      <c r="E37" s="33"/>
+      <c r="F37" s="33"/>
+      <c r="G37" s="33"/>
+      <c r="H37" s="34"/>
     </row>
     <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
@@ -8464,25 +8480,25 @@
       <c r="C41" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D41" s="32" t="s">
+      <c r="D41" s="38" t="s">
         <v>221</v>
       </c>
-      <c r="E41" s="33"/>
-      <c r="F41" s="33"/>
-      <c r="G41" s="33"/>
-      <c r="H41" s="34"/>
+      <c r="E41" s="39"/>
+      <c r="F41" s="39"/>
+      <c r="G41" s="39"/>
+      <c r="H41" s="40"/>
     </row>
     <row r="42" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="44" t="s">
+      <c r="D42" s="32" t="s">
         <v>257</v>
       </c>
-      <c r="E42" s="45"/>
-      <c r="F42" s="45"/>
-      <c r="G42" s="45"/>
-      <c r="H42" s="46"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="34"/>
     </row>
     <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
@@ -8500,25 +8516,25 @@
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
-      <c r="D44" s="44" t="s">
+      <c r="D44" s="32" t="s">
         <v>258</v>
       </c>
-      <c r="E44" s="45"/>
-      <c r="F44" s="45"/>
-      <c r="G44" s="45"/>
-      <c r="H44" s="46"/>
+      <c r="E44" s="33"/>
+      <c r="F44" s="33"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="34"/>
     </row>
     <row r="45" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
-      <c r="D45" s="44" t="s">
+      <c r="D45" s="32" t="s">
         <v>381</v>
       </c>
-      <c r="E45" s="45"/>
-      <c r="F45" s="45"/>
-      <c r="G45" s="45"/>
-      <c r="H45" s="46"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="33"/>
+      <c r="H45" s="34"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
@@ -8530,37 +8546,37 @@
       <c r="C46" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D46" s="32" t="s">
+      <c r="D46" s="38" t="s">
         <v>259</v>
       </c>
-      <c r="E46" s="33"/>
-      <c r="F46" s="33"/>
-      <c r="G46" s="33"/>
-      <c r="H46" s="34"/>
+      <c r="E46" s="39"/>
+      <c r="F46" s="39"/>
+      <c r="G46" s="39"/>
+      <c r="H46" s="40"/>
     </row>
     <row r="47" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="44" t="s">
+      <c r="D47" s="32" t="s">
         <v>138</v>
       </c>
-      <c r="E47" s="45"/>
-      <c r="F47" s="45"/>
-      <c r="G47" s="45"/>
-      <c r="H47" s="46"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="34"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
-      <c r="D48" s="44" t="s">
+      <c r="D48" s="32" t="s">
         <v>139</v>
       </c>
-      <c r="E48" s="45"/>
-      <c r="F48" s="45"/>
-      <c r="G48" s="45"/>
-      <c r="H48" s="46"/>
+      <c r="E48" s="33"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="33"/>
+      <c r="H48" s="34"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
@@ -8584,49 +8600,49 @@
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
-      <c r="D50" s="44" t="s">
+      <c r="D50" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="E50" s="45"/>
-      <c r="F50" s="45"/>
-      <c r="G50" s="45"/>
-      <c r="H50" s="46"/>
+      <c r="E50" s="33"/>
+      <c r="F50" s="33"/>
+      <c r="G50" s="33"/>
+      <c r="H50" s="34"/>
     </row>
     <row r="51" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="44" t="s">
+      <c r="D51" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
-      <c r="G51" s="45"/>
-      <c r="H51" s="46"/>
+      <c r="E51" s="33"/>
+      <c r="F51" s="33"/>
+      <c r="G51" s="33"/>
+      <c r="H51" s="34"/>
     </row>
     <row r="52" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="44" t="s">
+      <c r="D52" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="E52" s="45"/>
-      <c r="F52" s="45"/>
-      <c r="G52" s="45"/>
-      <c r="H52" s="46"/>
+      <c r="E52" s="33"/>
+      <c r="F52" s="33"/>
+      <c r="G52" s="33"/>
+      <c r="H52" s="34"/>
     </row>
     <row r="53" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
-      <c r="D53" s="44" t="s">
+      <c r="D53" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="E53" s="45"/>
-      <c r="F53" s="45"/>
-      <c r="G53" s="45"/>
-      <c r="H53" s="46"/>
+      <c r="E53" s="33"/>
+      <c r="F53" s="33"/>
+      <c r="G53" s="33"/>
+      <c r="H53" s="34"/>
     </row>
     <row r="54" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
@@ -8721,25 +8737,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -8769,37 +8785,37 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>319</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>320</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="53"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -8811,13 +8827,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -8847,37 +8863,37 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>321</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>322</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -8901,13 +8917,13 @@
       <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="40"/>
     </row>
     <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -8979,25 +8995,25 @@
       <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40"/>
     </row>
     <row r="22" spans="1:8" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="51" t="s">
+      <c r="D22" s="48" t="s">
         <v>325</v>
       </c>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="53"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -9033,13 +9049,13 @@
       <c r="C25" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D25" s="32" t="s">
+      <c r="D25" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="34"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="40"/>
     </row>
     <row r="26" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
@@ -9099,13 +9115,13 @@
       <c r="C30" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D30" s="32" t="s">
+      <c r="D30" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="34"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="40"/>
     </row>
     <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
@@ -9165,13 +9181,13 @@
       <c r="C35" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D35" s="32" t="s">
+      <c r="D35" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="34"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="39"/>
+      <c r="H35" s="40"/>
     </row>
     <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
@@ -9207,13 +9223,13 @@
       <c r="C38" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D38" s="32" t="s">
+      <c r="D38" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="33"/>
-      <c r="H38" s="34"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="40"/>
     </row>
     <row r="39" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
@@ -9346,25 +9362,25 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -9394,37 +9410,37 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>319</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="53"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>270</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="53"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -9436,13 +9452,13 @@
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
@@ -9472,49 +9488,49 @@
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="51" t="s">
         <v>298</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="43"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="53"/>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>272</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="51" t="s">
         <v>171</v>
       </c>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="43"/>
+      <c r="E14" s="52"/>
+      <c r="F14" s="52"/>
+      <c r="G14" s="52"/>
+      <c r="H14" s="53"/>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
@@ -9538,13 +9554,13 @@
       <c r="C16" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="34"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="40"/>
     </row>
     <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
@@ -9574,49 +9590,49 @@
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="40"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="47"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="51" t="s">
         <v>327</v>
       </c>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="43"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="53"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="51" t="s">
         <v>328</v>
       </c>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="43"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="53"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="51" t="s">
         <v>142</v>
       </c>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="43"/>
+      <c r="E22" s="52"/>
+      <c r="F22" s="52"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="53"/>
     </row>
     <row r="23" spans="1:8" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -9640,13 +9656,13 @@
       <c r="C24" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D24" s="32" t="s">
+      <c r="D24" s="38" t="s">
         <v>173</v>
       </c>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="34"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="40"/>
     </row>
     <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
@@ -9676,37 +9692,37 @@
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="38" t="s">
+      <c r="D27" s="45" t="s">
         <v>176</v>
       </c>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="40"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="47"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="51" t="s">
         <v>329</v>
       </c>
-      <c r="E28" s="42"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42"/>
-      <c r="H28" s="43"/>
+      <c r="E28" s="52"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="52"/>
+      <c r="H28" s="53"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="51" t="s">
         <v>330</v>
       </c>
-      <c r="E29" s="42"/>
-      <c r="F29" s="42"/>
-      <c r="G29" s="42"/>
-      <c r="H29" s="43"/>
+      <c r="E29" s="52"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="52"/>
+      <c r="H29" s="53"/>
     </row>
     <row r="30" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -9730,13 +9746,13 @@
       <c r="C31" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D31" s="32" t="s">
+      <c r="D31" s="38" t="s">
         <v>177</v>
       </c>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="34"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="39"/>
+      <c r="G31" s="39"/>
+      <c r="H31" s="40"/>
     </row>
     <row r="32" spans="1:8" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -9796,13 +9812,13 @@
       <c r="C36" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D36" s="32" t="s">
+      <c r="D36" s="38" t="s">
         <v>181</v>
       </c>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="34"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
+      <c r="H36" s="40"/>
     </row>
     <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
@@ -9832,25 +9848,25 @@
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="44" t="s">
+      <c r="D39" s="32" t="s">
         <v>332</v>
       </c>
-      <c r="E39" s="45"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="45"/>
-      <c r="H39" s="46"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="33"/>
+      <c r="H39" s="34"/>
     </row>
     <row r="40" spans="1:8" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="44" t="s">
+      <c r="D40" s="32" t="s">
         <v>333</v>
       </c>
-      <c r="E40" s="45"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="46"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
+      <c r="H40" s="34"/>
     </row>
     <row r="41" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -9874,13 +9890,13 @@
       <c r="C42" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D42" s="32" t="s">
+      <c r="D42" s="38" t="s">
         <v>182</v>
       </c>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="34"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="39"/>
+      <c r="G42" s="39"/>
+      <c r="H42" s="40"/>
     </row>
     <row r="43" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
@@ -9952,13 +9968,13 @@
       <c r="C48" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D48" s="32" t="s">
+      <c r="D48" s="38" t="s">
         <v>141</v>
       </c>
-      <c r="E48" s="33"/>
-      <c r="F48" s="33"/>
-      <c r="G48" s="33"/>
-      <c r="H48" s="34"/>
+      <c r="E48" s="39"/>
+      <c r="F48" s="39"/>
+      <c r="G48" s="39"/>
+      <c r="H48" s="40"/>
     </row>
     <row r="49" spans="1:10" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
@@ -10105,13 +10121,13 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="12"/>
@@ -10141,13 +10157,13 @@
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
-      <c r="D4" s="48" t="s">
+      <c r="D4" s="42" t="s">
         <v>191</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="50"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -10159,13 +10175,13 @@
       <c r="C5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="34"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="40"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="12"/>
@@ -10297,13 +10313,13 @@
       <c r="C16" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="38" t="s">
         <v>76</v>
       </c>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="34"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="40"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="12"/>
@@ -10333,13 +10349,13 @@
       <c r="A19" s="12"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="40"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="47"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="12"/>
@@ -10387,25 +10403,25 @@
       <c r="C23" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D23" s="32" t="s">
+      <c r="D23" s="38" t="s">
         <v>77</v>
       </c>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="34"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="40"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="12"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="51" t="s">
+      <c r="D24" s="48" t="s">
         <v>192</v>
       </c>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="53"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="50"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="12"/>
@@ -10465,13 +10481,13 @@
       <c r="C29" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="38" t="s">
         <v>78</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="34"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="40"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="12"/>
@@ -10531,13 +10547,13 @@
       <c r="C34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D34" s="32" t="s">
+      <c r="D34" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="34"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="40"/>
     </row>
     <row r="35" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="12"/>
@@ -10597,13 +10613,13 @@
       <c r="C39" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D39" s="32" t="s">
+      <c r="D39" s="38" t="s">
         <v>80</v>
       </c>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-      <c r="G39" s="33"/>
-      <c r="H39" s="34"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="39"/>
+      <c r="G39" s="39"/>
+      <c r="H39" s="40"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="12"/>
@@ -10735,13 +10751,13 @@
       <c r="C50" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D50" s="32" t="s">
+      <c r="D50" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="E50" s="33"/>
-      <c r="F50" s="33"/>
-      <c r="G50" s="33"/>
-      <c r="H50" s="34"/>
+      <c r="E50" s="39"/>
+      <c r="F50" s="39"/>
+      <c r="G50" s="39"/>
+      <c r="H50" s="40"/>
     </row>
     <row r="51" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="12"/>

</xml_diff>